<commit_message>
fix(E25): separate normalization and pooling dilution wells
</commit_message>
<xml_diff>
--- a/产品信息/PTseq_v12_source_reagent_loading_table.xlsx
+++ b/产品信息/PTseq_v12_source_reagent_loading_table.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="试剂分装" sheetId="1" r:id="R4fe3334e71cf4b21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="代码消耗" sheetId="2" r:id="Rc981d402aa144898"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="计算明细" sheetId="3" r:id="R2b4b7ed99a27465f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="4" r:id="Rf91af93b8cc844df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="均一化设计" sheetId="5" r:id="Rba57b8e356b44d8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E25_DNB试剂" sheetId="6" r:id="R8f49c520569b4e27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G99_DNB试剂" sheetId="7" r:id="Ra402c5abfaa544d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="200_2000_DNB试剂" sheetId="8" r:id="R08d6f3474f3e4b7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="试剂分装" sheetId="1" r:id="R692ef27aa6874db8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="代码消耗" sheetId="2" r:id="R822b5f8f23f241a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="计算明细" sheetId="3" r:id="Rb00ab7d8dbf749f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="4" r:id="R7a4536703e544f89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="均一化设计" sheetId="5" r:id="R3cf762c1d7b445fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E25_DNB试剂" sheetId="6" r:id="R254d130ccf414b09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G99_DNB试剂" sheetId="7" r:id="R8cd8d43457334113"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="200_2000_DNB试剂" sheetId="8" r:id="R4c0bcfa6acc24495"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3680,7 +3680,7 @@
         </x:is>
       </x:c>
       <x:c r="B18" t="str">
-        <x:v>POS8 Col1-4为提取原液，Col7-10为均一化产物；POS14 Col7-10为提取定量管，Col1-4保留最终文库定量；POS30保持为空置中转位。</x:v>
+        <x:v>POS8 Col1-4为提取原液，Col5-8为均一化产物，Col9-12为pooling预稀释；POS14 Col7-10为提取定量管，Col1-4保留最终文库定量；POS30保持为空置中转位。</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -4086,7 +4086,7 @@
         </x:is>
       </x:c>
       <x:c r="C14" s="13" t="str">
-        <x:v>Col7-10</x:v>
+        <x:v>Col5-8</x:v>
       </x:c>
       <x:c r="D14" s="7" t="n"/>
       <x:c r="E14" s="12" t="inlineStr">
@@ -4101,18 +4101,14 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="15" customHeight="1">
-      <x:c r="A15" s="12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">POS14</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B15" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">提取产物定量管</x:t>
-        </x:is>
+      <x:c r="A15" s="12" t="str">
+        <x:v>POS8</x:v>
+      </x:c>
+      <x:c r="B15" s="14" t="str">
+        <x:v>pooling 预稀释</x:v>
       </x:c>
       <x:c r="C15" s="13" t="str">
-        <x:v>Col7-10</x:v>
+        <x:v>Col9-12</x:v>
       </x:c>
       <x:c r="D15" s="7" t="n"/>
       <x:c r="E15" s="15" t="inlineStr">
@@ -4134,11 +4130,11 @@
       </x:c>
       <x:c r="B16" s="14" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">最终文库定量管</x:t>
+          <x:t xml:space="preserve">提取产物定量管</x:t>
         </x:is>
       </x:c>
       <x:c r="C16" s="13" t="str">
-        <x:v>Col1-4</x:v>
+        <x:v>Col7-10</x:v>
       </x:c>
       <x:c r="D16" s="7" t="n"/>
       <x:c r="E16" s="7" t="n"/>
@@ -4147,25 +4143,35 @@
     <x:row r="17" ht="15" customHeight="1">
       <x:c r="A17" s="12" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">POS24 A2</x:t>
+          <x:t xml:space="preserve">POS14</x:t>
         </x:is>
       </x:c>
       <x:c r="B17" s="14" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">均一化无核酸水</x:t>
+          <x:t xml:space="preserve">最终文库定量管</x:t>
         </x:is>
       </x:c>
       <x:c r="C17" s="13" t="str">
-        <x:v>8 mL管</x:v>
+        <x:v>Col1-4</x:v>
       </x:c>
       <x:c r="D17" s="7" t="n"/>
       <x:c r="E17" s="7" t="n"/>
       <x:c r="F17" s="7" t="n"/>
     </x:row>
     <x:row r="18" ht="15" customHeight="1">
-      <x:c r="A18" s="15"/>
-      <x:c r="B18" s="16"/>
-      <x:c r="C18" s="17"/>
+      <x:c r="A18" s="15" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">POS24 A2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" s="16" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">均一化无核酸水</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="17" t="str">
+        <x:v>8 mL管</x:v>
+      </x:c>
       <x:c r="D18" s="7" t="n"/>
       <x:c r="E18" s="7" t="n"/>
       <x:c r="F18" s="7" t="n"/>

</xml_diff>

<commit_message>
fix(ptseq): apply test feedback and sync 20260908 package
</commit_message>
<xml_diff>
--- a/产品信息/PTseq_v12_source_reagent_loading_table.xlsx
+++ b/产品信息/PTseq_v12_source_reagent_loading_table.xlsx
@@ -701,33 +701,29 @@
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="D4" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">+6 µL</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2 × N</x:t>
-        </x:is>
+      <x:c r="D4" s="4" t="str">
+        <x:v>+10 µL</x:v>
+      </x:c>
+      <x:c r="E4" s="4" t="str">
+        <x:v>2 × N；加10 µL来源冗余后向上取整到10 µL</x:v>
       </x:c>
       <x:c r="F4" s="7" t="n">
-        <x:v>25</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G4" s="7" t="n">
-        <x:v>40</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="H4" s="7" t="n">
-        <x:v>55</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="I4" s="7" t="n">
-        <x:v>70</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="J4" s="7" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="K4" s="7" t="n">
-        <x:v>105</x:v>
+        <x:v>110</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
@@ -1000,11 +996,9 @@
         <x:v>1370</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="30" customHeight="1">
-      <x:c r="A11" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T2缓冲液总量</x:t>
-        </x:is>
+    <x:row r="11" ht="40" customHeight="1">
+      <x:c r="A11" s="4" t="str">
+        <x:v>T2缓冲液（其他路线）</x:v>
       </x:c>
       <x:c r="B11" s="4" t="inlineStr">
         <x:is>
@@ -1045,60 +1039,50 @@
         <x:v>5355</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="15" customHeight="1">
-      <x:c r="A12" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">磁珠总量</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B12" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">POS24 C1R1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C12" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">8 mL管</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D12" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">+400 µL</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E12" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TA磁珠 50 × 1.4 × N + LA磁珠 55 × N</x:t>
-        </x:is>
+    <x:row r="12" ht="40" customHeight="1">
+      <x:c r="A12" s="4" t="str">
+        <x:v>T2缓冲液（E25全流程）</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>POS24 C1R2</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="str">
+        <x:v>8 mL管</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="str">
+        <x:v>已含320 µL</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="str">
+        <x:v>1个DNB；N−1个非空白文库均8倍稀释，另含动态补液及来源冗余；32例按5000 µL备液</x:v>
       </x:c>
       <x:c r="F12" s="7" t="n">
-        <x:v>1400</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="G12" s="7" t="n">
         <x:v>2400</x:v>
       </x:c>
       <x:c r="H12" s="7" t="n">
-        <x:v>3400</x:v>
+        <x:v>3600</x:v>
       </x:c>
       <x:c r="I12" s="7" t="n">
-        <x:v>4400</x:v>
-      </x:c>
-      <x:c r="J12" s="7" t="n">
-        <x:v>5400</x:v>
-      </x:c>
-      <x:c r="K12" s="7" t="n">
-        <x:v>6400</x:v>
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="J12" s="7" t="str">
+        <x:v>/</x:v>
+      </x:c>
+      <x:c r="K12" s="7" t="str">
+        <x:v>/</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" customHeight="1">
       <x:c r="A13" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">矿物油</x:t>
+          <x:t xml:space="preserve">磁珠总量</x:t>
         </x:is>
       </x:c>
       <x:c r="B13" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">POS24 C3R1</x:t>
+          <x:t xml:space="preserve">POS24 C1R1</x:t>
         </x:is>
       </x:c>
       <x:c r="C13" s="4" t="inlineStr">
@@ -1108,255 +1092,300 @@
       </x:c>
       <x:c r="D13" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">+320 µL</x:t>
+          <x:t xml:space="preserve">+400 µL</x:t>
         </x:is>
       </x:c>
       <x:c r="E13" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">按当前代码逻辑计算矿物油预分装总量</x:t>
+          <x:t xml:space="preserve">TA磁珠 50 × 1.4 × N + LA磁珠 55 × N</x:t>
         </x:is>
       </x:c>
       <x:c r="F13" s="7" t="n">
-        <x:v>880</x:v>
+        <x:v>1400</x:v>
       </x:c>
       <x:c r="G13" s="7" t="n">
-        <x:v>1440</x:v>
+        <x:v>2400</x:v>
       </x:c>
       <x:c r="H13" s="7" t="n">
-        <x:v>2000</x:v>
+        <x:v>3400</x:v>
       </x:c>
       <x:c r="I13" s="7" t="n">
-        <x:v>2240</x:v>
+        <x:v>4400</x:v>
       </x:c>
       <x:c r="J13" s="7" t="n">
-        <x:v>2720</x:v>
+        <x:v>5400</x:v>
       </x:c>
       <x:c r="K13" s="7" t="n">
-        <x:v>3200</x:v>
+        <x:v>6400</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" customHeight="1">
       <x:c r="A14" s="4" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">矿物油</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">POS24 C3R1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">8 mL管</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">+320 µL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">按当前代码逻辑计算矿物油预分装总量</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F14" s="7" t="n">
+        <x:v>880</x:v>
+      </x:c>
+      <x:c r="G14" s="7" t="n">
+        <x:v>1440</x:v>
+      </x:c>
+      <x:c r="H14" s="7" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="I14" s="7" t="n">
+        <x:v>2240</x:v>
+      </x:c>
+      <x:c r="J14" s="7" t="n">
+        <x:v>2720</x:v>
+      </x:c>
+      <x:c r="K14" s="7" t="n">
+        <x:v>3200</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" customHeight="1">
+      <x:c r="A15" s="4" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve">80%乙醇</x:t>
         </x:is>
       </x:c>
-      <x:c r="B14" s="4" t="inlineStr">
+      <x:c r="B15" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS3 reservoir</x:t>
         </x:is>
       </x:c>
-      <x:c r="C14" s="4" t="inlineStr">
+      <x:c r="C15" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">50 mL储液槽</x:t>
         </x:is>
       </x:c>
-      <x:c r="D14" s="4" t="inlineStr">
+      <x:c r="D15" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">+3200 µL</x:t>
         </x:is>
       </x:c>
-      <x:c r="E14" s="4" t="inlineStr">
+      <x:c r="E15" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">195 × 5 × N</x:t>
         </x:is>
       </x:c>
-      <x:c r="F14" s="7" t="n">
+      <x:c r="F15" s="7" t="n">
         <x:v>11000</x:v>
       </x:c>
-      <x:c r="G14" s="7" t="n">
+      <x:c r="G15" s="7" t="n">
         <x:v>18800</x:v>
       </x:c>
-      <x:c r="H14" s="7" t="n">
+      <x:c r="H15" s="7" t="n">
         <x:v>26600</x:v>
       </x:c>
-      <x:c r="I14" s="7" t="n">
+      <x:c r="I15" s="7" t="n">
         <x:v>34400</x:v>
       </x:c>
-      <x:c r="J14" s="7" t="n">
+      <x:c r="J15" s="7" t="n">
         <x:v>42200</x:v>
       </x:c>
-      <x:c r="K14" s="7" t="n">
+      <x:c r="K15" s="7" t="n">
         <x:v>50000</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="15" customHeight="1">
-      <x:c r="A15" s="4" t="str">
+    <x:row r="16" ht="15" customHeight="1">
+      <x:c r="A16" s="4" t="str">
         <x:v>Qubit染液（G99/200/2000）</x:v>
       </x:c>
-      <x:c r="B15" s="4" t="inlineStr">
+      <x:c r="B16" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS4 C1R1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C15" s="4" t="inlineStr">
+      <x:c r="C16" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">50 mL储液槽</x:t>
         </x:is>
       </x:c>
-      <x:c r="D15" s="4" t="inlineStr">
+      <x:c r="D16" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">+6510 µL</x:t>
         </x:is>
       </x:c>
-      <x:c r="E15" s="4" t="str">
+      <x:c r="E16" s="4" t="str">
         <x:v>单轮定量：217.8 × N + 6510 µL试剂槽管底冗余，向上取1000 µL</x:v>
       </x:c>
-      <x:c r="F15" s="7" t="n">
+      <x:c r="F16" s="7" t="n">
         <x:f>CEILING(F$3*217.8+6510,1000)</x:f>
         <x:v>9000</x:v>
       </x:c>
-      <x:c r="G15" s="7" t="n">
+      <x:c r="G16" s="7" t="n">
         <x:f>CEILING(G$3*217.8+6510,1000)</x:f>
         <x:v>10000</x:v>
       </x:c>
-      <x:c r="H15" s="7" t="n">
+      <x:c r="H16" s="7" t="n">
         <x:f>CEILING(H$3*217.8+6510,1000)</x:f>
         <x:v>12000</x:v>
       </x:c>
-      <x:c r="I15" s="7" t="n">
+      <x:c r="I16" s="7" t="n">
         <x:f>CEILING(I$3*217.8+6510,1000)</x:f>
         <x:v>14000</x:v>
       </x:c>
-      <x:c r="J15" s="7" t="n">
+      <x:c r="J16" s="7" t="n">
         <x:f>CEILING(J$3*217.8+6510,1000)</x:f>
         <x:v>16000</x:v>
       </x:c>
-      <x:c r="K15" s="7" t="n">
+      <x:c r="K16" s="7" t="n">
         <x:f>CEILING(K$3*217.8+6510,1000)</x:f>
         <x:v>17000</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="35.75" customHeight="1">
-      <x:c r="A16" t="str">
+    <x:row r="17" ht="35.75" customHeight="1">
+      <x:c r="A17" t="str">
         <x:v>Qubit染液（E25全流程）</x:v>
       </x:c>
-      <x:c r="B16" t="str">
+      <x:c r="B17" t="str">
         <x:v>POS4 C1R1</x:v>
       </x:c>
-      <x:c r="C16" t="str">
+      <x:c r="C17" t="str">
         <x:v>50 mL储液槽</x:v>
       </x:c>
-      <x:c r="D16" t="str">
+      <x:c r="D17" t="str">
         <x:v>+6510 µL</x:v>
       </x:c>
-      <x:c r="E16" t="str">
+      <x:c r="E17" t="str">
         <x:v>两轮定量：2 × 217.8 × N + 6510 µL试剂槽管底冗余，向上取1000 µL</x:v>
       </x:c>
-      <x:c r="F16" t="n">
+      <x:c r="F17" t="n">
         <x:f>CEILING(F$3*217.8*2+6510,1000)</x:f>
         <x:v>10000</x:v>
       </x:c>
-      <x:c r="G16" t="n">
+      <x:c r="G17" t="n">
         <x:f>CEILING(G$3*217.8*2+6510,1000)</x:f>
         <x:v>14000</x:v>
       </x:c>
-      <x:c r="H16" t="n">
+      <x:c r="H17" t="n">
         <x:f>CEILING(H$3*217.8*2+6510,1000)</x:f>
         <x:v>17000</x:v>
       </x:c>
-      <x:c r="I16" t="n">
+      <x:c r="I17" t="n">
         <x:f>CEILING(I$3*217.8*2+6510,1000)</x:f>
         <x:v>21000</x:v>
       </x:c>
-      <x:c r="J16" t="str">
+      <x:c r="J17" t="str">
         <x:v>/</x:v>
       </x:c>
-      <x:c r="K16" t="str">
+      <x:c r="K17" t="str">
         <x:v>/</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="35.75" customHeight="1">
-      <x:c r="A17" t="str">
+    <x:row r="18" ht="35.75" customHeight="1">
+      <x:c r="A18" t="str">
         <x:v>无核酸酶水（E25全流程）</x:v>
       </x:c>
-      <x:c r="B17" t="str">
+      <x:c r="B18" t="str">
         <x:v>POS24 A2</x:v>
       </x:c>
-      <x:c r="C17" t="str">
+      <x:c r="C18" t="str">
         <x:v>8 mL管</x:v>
       </x:c>
-      <x:c r="D17" t="str">
+      <x:c r="D18" t="str">
         <x:v>+320 µL</x:v>
       </x:c>
-      <x:c r="E17" t="str">
+      <x:c r="E18" t="str">
         <x:v>最大代码消耗27 × N + 320 µL来源死体积，向上取10 µL</x:v>
       </x:c>
-      <x:c r="F17" t="n">
+      <x:c r="F18" t="n">
         <x:f>CEILING(F$3*27+320,10)</x:f>
         <x:v>540</x:v>
       </x:c>
-      <x:c r="G17" t="n">
+      <x:c r="G18" t="n">
         <x:f>CEILING(G$3*27+320,10)</x:f>
         <x:v>760</x:v>
       </x:c>
-      <x:c r="H17" t="n">
+      <x:c r="H18" t="n">
         <x:f>CEILING(H$3*27+320,10)</x:f>
         <x:v>970</x:v>
       </x:c>
-      <x:c r="I17" t="n">
+      <x:c r="I18" t="n">
         <x:f>CEILING(I$3*27+320,10)</x:f>
         <x:v>1190</x:v>
       </x:c>
-      <x:c r="J17" t="str">
+      <x:c r="J18" t="str">
         <x:v>/</x:v>
       </x:c>
-      <x:c r="K17" t="str">
+      <x:c r="K18" t="str">
         <x:v>/</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" t="inlineStr">
+    <x:row r="19">
+      <x:c r="A19" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">T12 空白对照</x:t>
         </x:is>
       </x:c>
-      <x:c r="B18" t="inlineStr">
+      <x:c r="B19" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 F1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C18" t="inlineStr">
+      <x:c r="C19" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="D18" t="inlineStr">
+      <x:c r="D19" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">+6 µL</x:t>
         </x:is>
       </x:c>
-      <x:c r="E18" t="inlineStr">
+      <x:c r="E19" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">14 × 空白对照数量 + 6（质控类型为B的样本数）</x:t>
         </x:is>
       </x:c>
-      <x:c r="F18" t="inlineStr">
+      <x:c r="F19" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">14 × B + 6</x:t>
         </x:is>
       </x:c>
-      <x:c r="G18" t="inlineStr">
+      <x:c r="G19" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">14 × B + 6</x:t>
         </x:is>
       </x:c>
-      <x:c r="H18" t="inlineStr">
+      <x:c r="H19" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">14 × B + 6</x:t>
         </x:is>
       </x:c>
-      <x:c r="I18" t="inlineStr">
+      <x:c r="I19" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">14 × B + 6</x:t>
         </x:is>
       </x:c>
-      <x:c r="J18" t="inlineStr">
+      <x:c r="J19" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">14 × B + 6</x:t>
         </x:is>
       </x:c>
-      <x:c r="K18" t="inlineStr">
+      <x:c r="K19" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">14 × B + 6</x:t>
         </x:is>
@@ -1758,7 +1787,7 @@
         <x:v>2266.8</x:v>
       </x:c>
       <x:c r="H11" s="7" t="n">
-        <x:v>2964.4</x:v>
+        <x:v>2871.4</x:v>
       </x:c>
       <x:c r="I11" s="7" t="n">
         <x:v>3662</x:v>
@@ -2812,12 +2841,10 @@
         </x:is>
       </x:c>
       <x:c r="D34" s="27" t="n">
-        <x:v>429</x:v>
-      </x:c>
-      <x:c r="E34" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">第11列反应液总量 × 9/30；总量&gt;1421 µL时T2直接加入POS7 Col11。</x:t>
-        </x:is>
+        <x:v>336</x:v>
+      </x:c>
+      <x:c r="E34" s="4" t="str">
+        <x:v>32例时LA总量1430 µL超过1421 µL，T2直接加入POS7 Col11：8 × 140 × 9/30 = 336 µL。</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" customHeight="1">
@@ -3470,6 +3497,78 @@
         <x:is>
           <x:t xml:space="preserve">14 × 24 + (384 - 2 × 48) + 48 = 672；包含一半样本预稀释、pooling管补液上限及DNB孔补液上限。</x:t>
         </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="35.75" customHeight="1">
+      <x:c r="A64" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>E25 pooling T2预算</x:v>
+      </x:c>
+      <x:c r="C64" t="str">
+        <x:v>非空白文库全8倍稀释及动态补液</x:v>
+      </x:c>
+      <x:c r="D64" t="n">
+        <x:f>35*(A64-1)+(160-2*A64)+18</x:f>
+        <x:v>407</x:v>
+      </x:c>
+      <x:c r="E64" t="str">
+        <x:v>35 × (N−1) + (160−2×N) + 18；1个DNB，全部文库参与pooling；不含建库消耗和320 µL来源冗余。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="35.75" customHeight="1">
+      <x:c r="A65" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>E25 pooling T2预算</x:v>
+      </x:c>
+      <x:c r="C65" t="str">
+        <x:v>非空白文库全8倍稀释及动态补液</x:v>
+      </x:c>
+      <x:c r="D65" t="n">
+        <x:f>35*(A65-1)+(160-2*A65)+18</x:f>
+        <x:v>671</x:v>
+      </x:c>
+      <x:c r="E65" t="str">
+        <x:v>35 × (N−1) + (160−2×N) + 18；1个DNB，全部文库参与pooling；不含建库消耗和320 µL来源冗余。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="35.75" customHeight="1">
+      <x:c r="A66" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>E25 pooling T2预算</x:v>
+      </x:c>
+      <x:c r="C66" t="str">
+        <x:v>非空白文库全8倍稀释及动态补液</x:v>
+      </x:c>
+      <x:c r="D66" t="n">
+        <x:f>35*(A66-1)+(160-2*A66)+18</x:f>
+        <x:v>935</x:v>
+      </x:c>
+      <x:c r="E66" t="str">
+        <x:v>35 × (N−1) + (160−2×N) + 18；1个DNB，全部文库参与pooling；不含建库消耗和320 µL来源冗余。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="35.75" customHeight="1">
+      <x:c r="A67" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>E25 pooling T2预算</x:v>
+      </x:c>
+      <x:c r="C67" t="str">
+        <x:v>非空白文库全8倍稀释及动态补液</x:v>
+      </x:c>
+      <x:c r="D67" t="n">
+        <x:f>35*(A67-1)+(160-2*A67)+18</x:f>
+        <x:v>1199</x:v>
+      </x:c>
+      <x:c r="E67" t="str">
+        <x:v>35 × (N−1) + (160−2×N) + 18；1个DNB，全部文库参与pooling；不含建库消耗和320 µL来源冗余。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3516,7 +3615,7 @@
         </x:is>
       </x:c>
       <x:c r="B4" s="4" t="str">
-        <x:v>试剂分装主表覆盖 cDNA、TA、LA/PCR、两轮磁珠纯化、矿物油、乙醇和 Qubit 定量所需来源试剂；T2缓冲液额外包含G99 pooling预算。各测序平台makeDNB试剂见对应DNB试剂工作表。</x:v>
+        <x:v>试剂分装主表覆盖 cDNA、TA、LA/PCR、两轮磁珠纯化、矿物油、乙醇和 Qubit 定量所需来源试剂；T2缓冲液额外包含G99 pooling预算。各测序平台makeDNB试剂见对应DNB试剂工作表。 E25全流程T2装量单列，覆盖非空白文库全8倍预稀释场景。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" customHeight="1">
@@ -3538,7 +3637,7 @@
         </x:is>
       </x:c>
       <x:c r="B6" s="4" t="str">
-        <x:v>0.5 mL管通常 +6 µL，T4和T5例外为 +10 µL；2 mL管 +15 µL；8 mL管通常 +320 µL；磁珠总量特例 +400 µL；50 mL试剂槽按实际管底余量配置，80%乙醇 +3200 µL，Qubit染液 +6510 µL。</x:v>
+        <x:v>0.5 mL管通常 +6 µL，T4和T5例外为 +10 µL；2 mL管 +15 µL；8 mL管通常 +320 µL；磁珠总量特例 +400 µL；50 mL试剂槽按实际管底余量配置，80%乙醇 +3200 µL，Qubit染液 +6510 µL。 T1 cDNA引物来源冗余为10 µL，分装量向上取整到10 µL。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" customHeight="1">
@@ -3571,10 +3670,8 @@
           <x:t xml:space="preserve">T2缓冲液共用来源</x:t>
         </x:is>
       </x:c>
-      <x:c r="B9" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">POS24 C1R2合并建库阶段TA mix T2、POS7 Col7 T2中转量和LA/PCR mix T2；另按每批50%样本需要8倍预稀释，并覆盖pooling管与DNB孔动态补液上限，最后保留320 µL来源死体积。</x:t>
-        </x:is>
+      <x:c r="B9" s="4" t="str">
+        <x:v>POS24 C1R2合并建库阶段TA、POS7 Col7中转和LA/PCR的T2消耗。其他路线保留原G99 pooling预算；E25全流程按N−1个非空白文库全8倍稀释、1个DNB计入35 µL/孔和动态补液上限。分装1500/2400/3600/5000 µL均已含320 µL来源冗余。提取均一化无核酸酶水为独立来源，不计入T2。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" customHeight="1">
@@ -3781,6 +3878,14 @@
       </x:c>
       <x:c r="B27" t="str">
         <x:v>2026-08-28：按integration/e25-extraction-normalization更新E25提取产物定量与均一化；Qubit分装按对应定量轮次用量加6510 µL试剂槽管底冗余并向上取1000 µL；无核酸酶水使用POS24 A2 8 mL管，按27 × N + 320 µL并向上取10 µL；POS30保持为空置中转位。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>更新记录</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>2026-09-08：T1冗余调整为10 µL并统一取整；修正E25及200/2000 DNB酶分装量；增加E25全流程T2专用装量，32例为5000 µL；校正32例LA直接分装T2代码消耗为336 µL。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4296,22 +4401,20 @@
           <x:t xml:space="preserve">POS17 C2R5</x:t>
         </x:is>
       </x:c>
-      <x:c r="D5" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">40 × (D + 0.5)</x:t>
-        </x:is>
+      <x:c r="D5" s="20" t="str">
+        <x:v>40 × (D + 0.5) + 6</x:v>
       </x:c>
       <x:c r="E5" s="34" t="n">
-        <x:f>40*(E$3+0.5)</x:f>
-        <x:v>60</x:v>
+        <x:f>40*(E$3+0.5)+6</x:f>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="F5" s="34" t="n">
-        <x:f>40*(F$3+0.5)</x:f>
-        <x:v>100</x:v>
+        <x:f>40*(F$3+0.5)+6</x:f>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="G5" s="34" t="n">
-        <x:f>40*(G$3+0.5)</x:f>
-        <x:v>140</x:v>
+        <x:f>40*(G$3+0.5)+6</x:f>
+        <x:v>146</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
@@ -4330,22 +4433,20 @@
           <x:t xml:space="preserve">POS17 C3R5</x:t>
         </x:is>
       </x:c>
-      <x:c r="D6" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">5 × D + 10（按分装表）</x:t>
-        </x:is>
+      <x:c r="D6" s="20" t="str">
+        <x:v>4 × (D + 0.5)</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>5*E$3+10</x:f>
-        <x:v>15</x:v>
+        <x:f>4*(E$3+0.5)</x:f>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F6" s="34" t="n">
-        <x:f>5*F$3+10</x:f>
-        <x:v>20</x:v>
+        <x:f>4*(F$3+0.5)</x:f>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G6" s="34" t="n">
-        <x:f>5*G$3+10</x:f>
-        <x:v>25</x:v>
+        <x:f>4*(G$3+0.5)</x:f>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -4907,10 +5008,10 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="F7" s="34" t="n">
-        <x:v>120</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="G7" s="34" t="n">
-        <x:v>180</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="H7" s="34"/>
     </x:row>
@@ -4928,13 +5029,13 @@
         <x:v>按SOP表10-1手工分装</x:v>
       </x:c>
       <x:c r="E8" s="34" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F8" s="34" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G8" s="34" t="n">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="H8" s="34"/>
     </x:row>

</xml_diff>

<commit_message>
fix(docs): align Mix I loading volumes and sync active workbooks
</commit_message>
<xml_diff>
--- a/产品信息/PTseq_v12_source_reagent_loading_table.xlsx
+++ b/产品信息/PTseq_v12_source_reagent_loading_table.xlsx
@@ -4402,19 +4402,19 @@
         </x:is>
       </x:c>
       <x:c r="D5" s="20" t="str">
-        <x:v>40 × (D + 0.5) + 6</x:v>
+        <x:v>40×(D+0.5)+6，向上取10</x:v>
       </x:c>
       <x:c r="E5" s="34" t="n">
-        <x:f>40*(E$3+0.5)+6</x:f>
-        <x:v>66</x:v>
+        <x:f>CEILING(40*(E$3+0.5)+6,10)</x:f>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F5" s="34" t="n">
-        <x:f>40*(F$3+0.5)+6</x:f>
-        <x:v>106</x:v>
+        <x:f>CEILING(40*(F$3+0.5)+6,10)</x:f>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="G5" s="34" t="n">
-        <x:f>40*(G$3+0.5)+6</x:f>
-        <x:v>146</x:v>
+        <x:f>CEILING(40*(G$3+0.5)+6,10)</x:f>
+        <x:v>150</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">

</xml_diff>

<commit_message>
docs(ptseq): finalize dispensing and sync SOP bench images
Retain approved E25 T2 margins and SOP-authoritative loading tables, correct the figure reference, and sync three middle-platform bench images from the current SOP. Update the existing release record to the final 56-file delivery scope and cover-title SOP filename.
</commit_message>
<xml_diff>
--- a/产品信息/PTseq_v12_source_reagent_loading_table.xlsx
+++ b/产品信息/PTseq_v12_source_reagent_loading_table.xlsx
@@ -280,7 +280,7 @@
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -376,6 +376,39 @@
     </x:xf>
     <x:xf numFmtId="166" fontId="9" fillId="8" borderId="12" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="12" xfId="0" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="12" xfId="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="9" fillId="7" borderId="12" xfId="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="166" fontId="6" fillId="0" borderId="12" xfId="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="12" xfId="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="166" fontId="9" fillId="8" borderId="12" xfId="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -656,10 +689,8 @@
           <x:t xml:space="preserve">耗材类别</x:t>
         </x:is>
       </x:c>
-      <x:c r="D3" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">来源冗余</x:t>
-        </x:is>
+      <x:c r="D3" s="3" t="str">
+        <x:v>最低来源冗余</x:v>
       </x:c>
       <x:c r="E3" s="3" t="inlineStr">
         <x:is>
@@ -685,26 +716,24 @@
         <x:v>48</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="15" customHeight="1">
-      <x:c r="A4" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T1 cDNA引物</x:t>
-        </x:is>
+    <x:row r="4" ht="45" customHeight="1">
+      <x:c r="A4" s="46" t="str">
+        <x:v>T1 cDNA合成引物</x:v>
       </x:c>
       <x:c r="B4" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C1R1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C4" s="4" t="inlineStr">
+      <x:c r="C4" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="D4" s="4" t="str">
+      <x:c r="D4" s="46" t="str">
         <x:v>+10 µL</x:v>
       </x:c>
-      <x:c r="E4" s="4" t="str">
+      <x:c r="E4" s="46" t="str">
         <x:v>2 × N；加10 µL来源冗余后向上取整到10 µL</x:v>
       </x:c>
       <x:c r="F4" s="7" t="n">
@@ -726,31 +755,27 @@
         <x:v>110</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T2 cDNA缓冲液</x:t>
-        </x:is>
+    <x:row r="5" ht="45" customHeight="1">
+      <x:c r="A5" s="46" t="str">
+        <x:v>T2 一链合成缓冲液</x:v>
       </x:c>
       <x:c r="B5" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C2R1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C5" s="4" t="inlineStr">
+      <x:c r="C5" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="D5" s="4" t="inlineStr">
+      <x:c r="D5" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">+6 µL</x:t>
         </x:is>
       </x:c>
-      <x:c r="E5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">第9列反应液总量 / 2；&gt;16通量含2个完整POS7中转孔的上游冗余</x:t>
-        </x:is>
+      <x:c r="E5" s="46" t="str">
+        <x:v>第9列反应液总量 / 2 + 6 µL，向上取10 µL；分装量按SOP表9。</x:v>
       </x:c>
       <x:c r="F5" s="7" t="n">
         <x:v>30</x:v>
@@ -759,43 +784,39 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="H5" s="7" t="n">
-        <x:v>175</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="I5" s="7" t="n">
-        <x:v>195</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="J5" s="7" t="n">
-        <x:v>215</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="K5" s="7" t="n">
-        <x:v>235</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="30" customHeight="1">
-      <x:c r="A6" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T3 cDNA酶</x:t>
-        </x:is>
+        <x:v>240</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="45" customHeight="1">
+      <x:c r="A6" s="46" t="str">
+        <x:v>T3 一链合成酶</x:v>
       </x:c>
       <x:c r="B6" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C3R1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C6" s="4" t="inlineStr">
+      <x:c r="C6" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="D6" s="4" t="inlineStr">
+      <x:c r="D6" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">+6 µL</x:t>
         </x:is>
       </x:c>
-      <x:c r="E6" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">第9列反应液总量 / 2；&gt;16通量含2个完整POS7中转孔的上游冗余</x:t>
-        </x:is>
+      <x:c r="E6" s="46" t="str">
+        <x:v>第9列反应液总量 / 2 + 6 µL，向上取10 µL；分装量按SOP表9。</x:v>
       </x:c>
       <x:c r="F6" s="7" t="n">
         <x:v>30</x:v>
@@ -804,43 +825,37 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="H6" s="7" t="n">
-        <x:v>175</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="I6" s="7" t="n">
-        <x:v>195</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="J6" s="7" t="n">
-        <x:v>215</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="K6" s="7" t="n">
-        <x:v>235</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T4 TA缓冲液</x:t>
-        </x:is>
+        <x:v>240</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="45" customHeight="1">
+      <x:c r="A7" s="46" t="str">
+        <x:v>T4 靶向扩增缓冲液</x:v>
       </x:c>
       <x:c r="B7" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C1R2</x:t>
         </x:is>
       </x:c>
-      <x:c r="C7" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2 mL管</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D7" s="4" t="inlineStr">
+      <x:c r="C7" s="46" t="str">
+        <x:v>2.0 mL冻存管</x:v>
+      </x:c>
+      <x:c r="D7" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">+10 µL</x:t>
         </x:is>
       </x:c>
-      <x:c r="E7" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">第10列反应液总量 × 5/15；&gt;16通量含2个完整POS7中转孔的上游冗余</x:t>
-        </x:is>
+      <x:c r="E7" s="46" t="str">
+        <x:v>第10列反应液总量 × 5/15 + 10 µL，向上取10 µL；分装量按SOP表9。</x:v>
       </x:c>
       <x:c r="F7" s="7" t="n">
         <x:v>60</x:v>
@@ -849,65 +864,61 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="H7" s="7" t="n">
-        <x:v>235</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="I7" s="7" t="n">
-        <x:v>285</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="J7" s="7" t="n">
-        <x:v>335</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="K7" s="7" t="n">
-        <x:v>385</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="30" customHeight="1">
-      <x:c r="A8" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T5 TA酶</x:t>
-        </x:is>
+        <x:v>390</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="45" customHeight="1">
+      <x:c r="A8" s="46" t="str">
+        <x:v>T5 靶向扩增酶</x:v>
       </x:c>
       <x:c r="B8" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C2R2</x:t>
         </x:is>
       </x:c>
-      <x:c r="C8" s="4" t="inlineStr">
+      <x:c r="C8" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="D8" s="4" t="inlineStr">
+      <x:c r="D8" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">+10 µL</x:t>
         </x:is>
       </x:c>
-      <x:c r="E8" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">第10列反应液总量 × 3/15；&gt;16通量含2个完整POS7中转孔的上游冗余</x:t>
-        </x:is>
+      <x:c r="E8" s="46" t="str">
+        <x:v>第10列反应液总量 × 3/15 + 10 µL，向上取10 µL；分装量按SOP表9。</x:v>
       </x:c>
       <x:c r="F8" s="7" t="n">
         <x:v>40</x:v>
       </x:c>
       <x:c r="G8" s="7" t="n">
-        <x:v>65</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H8" s="7" t="n">
-        <x:v>145</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="I8" s="7" t="n">
-        <x:v>175</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="J8" s="7" t="n">
-        <x:v>205</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="K8" s="7" t="n">
-        <x:v>235</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="30" customHeight="1">
-      <x:c r="A9" s="4" t="inlineStr">
+        <x:v>240</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="45" customHeight="1">
+      <x:c r="A9" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">T8 UDG酶</x:t>
         </x:is>
@@ -917,20 +928,16 @@
           <x:t xml:space="preserve">POS17 C2R3</x:t>
         </x:is>
       </x:c>
-      <x:c r="C9" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2 mL管</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D9" s="4" t="inlineStr">
+      <x:c r="C9" s="46" t="str">
+        <x:v>2.0 mL冻存管</x:v>
+      </x:c>
+      <x:c r="D9" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">无源管冗余；手工预置到C2R3</x:t>
         </x:is>
       </x:c>
-      <x:c r="E9" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">第11列反应液总量 × 1/30；总量&gt;1421 µL时C2R3只配置T7+T8</x:t>
-        </x:is>
+      <x:c r="E9" s="46" t="str">
+        <x:v>第11列反应液总量 × 1/30，向上取1 µL；手工预置C2R3，分装量按SOP表9。</x:v>
       </x:c>
       <x:c r="F9" s="7" t="n">
         <x:v>9</x:v>
@@ -939,49 +946,41 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="H9" s="7" t="n">
-        <x:v>37.67</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="I9" s="7" t="n">
-        <x:v>47.67</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="J9" s="7" t="n">
-        <x:v>57.67</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="K9" s="7" t="n">
-        <x:v>67.67</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="30" customHeight="1">
-      <x:c r="A10" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T7 LA/PCR Mix</x:t>
-        </x:is>
+        <x:v>68</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="45" customHeight="1">
+      <x:c r="A10" s="46" t="str">
+        <x:v>T7 PCR Mix</x:v>
       </x:c>
       <x:c r="B10" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C1R3</x:t>
         </x:is>
       </x:c>
-      <x:c r="C10" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2 mL管</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D10" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">+15 µL，向上取5 µL</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E10" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">第11列反应液总量 × 20/30 + 源管冗余；总量&gt;1421 µL时C2R3只配置T7+T8</x:t>
-        </x:is>
+      <x:c r="C10" s="46" t="str">
+        <x:v>2.0 mL冻存管</x:v>
+      </x:c>
+      <x:c r="D10" s="46" t="str">
+        <x:v>+15 µL，向上取10 µL</x:v>
+      </x:c>
+      <x:c r="E10" s="46" t="str">
+        <x:v>第11列反应液总量 × 20/30 + 15 µL，向上取10 µL；分装量按SOP表9。</x:v>
       </x:c>
       <x:c r="F10" s="7" t="n">
-        <x:v>195</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="G10" s="7" t="n">
-        <x:v>355</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="H10" s="7" t="n">
         <x:v>770</x:v>
@@ -996,35 +995,31 @@
         <x:v>1370</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="40" customHeight="1">
-      <x:c r="A11" s="4" t="str">
-        <x:v>T2缓冲液（其他路线）</x:v>
+    <x:row r="11" ht="70" customHeight="1">
+      <x:c r="A11" s="46" t="str">
+        <x:v>T2溶解液（前处理建库及G99/200/2000全流程）</x:v>
       </x:c>
       <x:c r="B11" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS24 C1R2</x:t>
         </x:is>
       </x:c>
-      <x:c r="C11" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">8 mL管</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D11" s="4" t="inlineStr">
+      <x:c r="C11" s="46" t="str">
+        <x:v>8.0 mL冻存管</x:v>
+      </x:c>
+      <x:c r="D11" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">+320 µL</x:t>
         </x:is>
       </x:c>
-      <x:c r="E11" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">建库阶段T2 + G99 pooling预算（50%样本各14 µL预稀释，并覆盖pooling管及DNB孔动态补液上限）+ 320 µL来源死体积</x:t>
-        </x:is>
+      <x:c r="E11" s="46" t="str">
+        <x:v>建库阶段T2消耗 + G99 pooling预算 + 320 µL，向上取10 µL；适用流程和分装量按SOP表9。</x:v>
       </x:c>
       <x:c r="F11" s="7" t="n">
         <x:v>1480</x:v>
       </x:c>
       <x:c r="G11" s="7" t="n">
-        <x:v>2185</x:v>
+        <x:v>2190</x:v>
       </x:c>
       <x:c r="H11" s="7" t="n">
         <x:v>3140</x:v>
@@ -1033,36 +1028,36 @@
         <x:v>3880</x:v>
       </x:c>
       <x:c r="J11" s="7" t="n">
-        <x:v>4615</x:v>
+        <x:v>4620</x:v>
       </x:c>
       <x:c r="K11" s="7" t="n">
-        <x:v>5355</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="40" customHeight="1">
-      <x:c r="A12" s="4" t="str">
-        <x:v>T2缓冲液（E25全流程）</x:v>
+        <x:v>5360</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="70" customHeight="1">
+      <x:c r="A12" s="46" t="str">
+        <x:v>T2溶解液（E25全流程）</x:v>
       </x:c>
       <x:c r="B12" s="4" t="str">
         <x:v>POS24 C1R2</x:v>
       </x:c>
-      <x:c r="C12" s="4" t="str">
-        <x:v>8 mL管</x:v>
-      </x:c>
-      <x:c r="D12" s="4" t="str">
-        <x:v>已含320 µL</x:v>
-      </x:c>
-      <x:c r="E12" s="4" t="str">
-        <x:v>1个DNB；N−1个非空白文库均8倍稀释，另含动态补液及来源冗余；32例按5000 µL备液</x:v>
+      <x:c r="C12" s="46" t="str">
+        <x:v>8.0 mL冻存管</x:v>
+      </x:c>
+      <x:c r="D12" s="46" t="str">
+        <x:v>已含320 µL来源冗余及额外600 µL</x:v>
+      </x:c>
+      <x:c r="E12" s="46" t="str">
+        <x:v>1个DNB；N−1个非空白文库均8倍稀释；建库消耗、动态补液及320 µL来源冗余合计向上取100 µL，再加600 µL。</x:v>
       </x:c>
       <x:c r="F12" s="7" t="n">
-        <x:v>1500</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G12" s="7" t="n">
-        <x:v>2400</x:v>
+        <x:v>3000</x:v>
       </x:c>
       <x:c r="H12" s="7" t="n">
-        <x:v>3600</x:v>
+        <x:v>4200</x:v>
       </x:c>
       <x:c r="I12" s="7" t="n">
         <x:v>5000</x:v>
@@ -1074,28 +1069,24 @@
         <x:v>/</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="15" customHeight="1">
-      <x:c r="A13" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">磁珠总量</x:t>
-        </x:is>
+    <x:row r="13" ht="45" customHeight="1">
+      <x:c r="A13" s="46" t="str">
+        <x:v>T1磁珠</x:v>
       </x:c>
       <x:c r="B13" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS24 C1R1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C13" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">8 mL管</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D13" s="4" t="inlineStr">
+      <x:c r="C13" s="46" t="str">
+        <x:v>8.0 mL冻存管</x:v>
+      </x:c>
+      <x:c r="D13" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">+400 µL</x:t>
         </x:is>
       </x:c>
-      <x:c r="E13" s="4" t="inlineStr">
+      <x:c r="E13" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">TA磁珠 50 × 1.4 × N + LA磁珠 55 × N</x:t>
         </x:is>
@@ -1119,8 +1110,8 @@
         <x:v>6400</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="15" customHeight="1">
-      <x:c r="A14" s="4" t="inlineStr">
+    <x:row r="14" ht="45" customHeight="1">
+      <x:c r="A14" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">矿物油</x:t>
         </x:is>
@@ -1130,17 +1121,15 @@
           <x:t xml:space="preserve">POS24 C3R1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C14" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">8 mL管</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D14" s="4" t="inlineStr">
+      <x:c r="C14" s="46" t="str">
+        <x:v>8.0 mL冻存管</x:v>
+      </x:c>
+      <x:c r="D14" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">+320 µL</x:t>
         </x:is>
       </x:c>
-      <x:c r="E14" s="4" t="inlineStr">
+      <x:c r="E14" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">按当前代码逻辑计算矿物油预分装总量</x:t>
         </x:is>
@@ -1164,8 +1153,8 @@
         <x:v>3200</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="15" customHeight="1">
-      <x:c r="A15" s="4" t="inlineStr">
+    <x:row r="15" ht="45" customHeight="1">
+      <x:c r="A15" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">80%乙醇</x:t>
         </x:is>
@@ -1175,60 +1164,54 @@
           <x:t xml:space="preserve">POS3 reservoir</x:t>
         </x:is>
       </x:c>
-      <x:c r="C15" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">50 mL储液槽</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D15" s="4" t="inlineStr">
+      <x:c r="C15" s="46" t="str">
+        <x:v>50 mL试剂槽</x:v>
+      </x:c>
+      <x:c r="D15" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">+3200 µL</x:t>
         </x:is>
       </x:c>
-      <x:c r="E15" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">195 × 5 × N</x:t>
-        </x:is>
+      <x:c r="E15" s="46" t="str">
+        <x:v>195 × 5 × N + 3200 µL，向上取1000 µL；按SOP表9为11/19/27/35/43/50 mL。</x:v>
       </x:c>
       <x:c r="F15" s="7" t="n">
         <x:v>11000</x:v>
       </x:c>
       <x:c r="G15" s="7" t="n">
-        <x:v>18800</x:v>
+        <x:v>19000</x:v>
       </x:c>
       <x:c r="H15" s="7" t="n">
-        <x:v>26600</x:v>
+        <x:v>27000</x:v>
       </x:c>
       <x:c r="I15" s="7" t="n">
-        <x:v>34400</x:v>
+        <x:v>35000</x:v>
       </x:c>
       <x:c r="J15" s="7" t="n">
-        <x:v>42200</x:v>
+        <x:v>43000</x:v>
       </x:c>
       <x:c r="K15" s="7" t="n">
         <x:v>50000</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="15" customHeight="1">
-      <x:c r="A16" s="4" t="str">
-        <x:v>Qubit染液（G99/200/2000）</x:v>
+    <x:row r="16" ht="70" customHeight="1">
+      <x:c r="A16" s="46" t="str">
+        <x:v>Qubit染液（G99、200、2000全流程，前处理建库）</x:v>
       </x:c>
       <x:c r="B16" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS4 C1R1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C16" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">50 mL储液槽</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D16" s="4" t="inlineStr">
+      <x:c r="C16" s="46" t="str">
+        <x:v>50 mL避光试剂槽</x:v>
+      </x:c>
+      <x:c r="D16" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">+6510 µL</x:t>
         </x:is>
       </x:c>
-      <x:c r="E16" s="4" t="str">
+      <x:c r="E16" s="46" t="str">
         <x:v>单轮定量：217.8 × N + 6510 µL试剂槽管底冗余，向上取1000 µL</x:v>
       </x:c>
       <x:c r="F16" s="7" t="n">
@@ -1256,20 +1239,20 @@
         <x:v>17000</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="35.75" customHeight="1">
-      <x:c r="A17" t="str">
-        <x:v>Qubit染液（E25全流程）</x:v>
+    <x:row r="17" ht="70" customHeight="1">
+      <x:c r="A17" t="str" s="45">
+        <x:v>Qubit染液（E25全流程，前处理建库）</x:v>
       </x:c>
       <x:c r="B17" t="str">
         <x:v>POS4 C1R1</x:v>
       </x:c>
-      <x:c r="C17" t="str">
-        <x:v>50 mL储液槽</x:v>
-      </x:c>
-      <x:c r="D17" t="str">
+      <x:c r="C17" t="str" s="45">
+        <x:v>50 mL避光试剂槽</x:v>
+      </x:c>
+      <x:c r="D17" t="str" s="45">
         <x:v>+6510 µL</x:v>
       </x:c>
-      <x:c r="E17" t="str">
+      <x:c r="E17" t="str" s="45">
         <x:v>两轮定量：2 × 217.8 × N + 6510 µL试剂槽管底冗余，向上取1000 µL</x:v>
       </x:c>
       <x:c r="F17" t="n">
@@ -1295,20 +1278,20 @@
         <x:v>/</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="35.75" customHeight="1">
-      <x:c r="A18" t="str">
+    <x:row r="18" ht="45" customHeight="1">
+      <x:c r="A18" t="str" s="45">
         <x:v>无核酸酶水（E25全流程）</x:v>
       </x:c>
       <x:c r="B18" t="str">
         <x:v>POS24 A2</x:v>
       </x:c>
-      <x:c r="C18" t="str">
-        <x:v>8 mL管</x:v>
-      </x:c>
-      <x:c r="D18" t="str">
+      <x:c r="C18" t="str" s="45">
+        <x:v>8.0 mL冻存管</x:v>
+      </x:c>
+      <x:c r="D18" t="str" s="45">
         <x:v>+320 µL</x:v>
       </x:c>
-      <x:c r="E18" t="str">
+      <x:c r="E18" t="str" s="45">
         <x:v>最大代码消耗27 × N + 320 µL来源死体积，向上取10 µL</x:v>
       </x:c>
       <x:c r="F18" t="n">
@@ -1334,8 +1317,8 @@
         <x:v>/</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" t="inlineStr">
+    <x:row r="19" ht="45" customHeight="1">
+      <x:c r="A19" t="inlineStr" s="45">
         <x:is>
           <x:t xml:space="preserve">T12 空白对照</x:t>
         </x:is>
@@ -1345,47 +1328,45 @@
           <x:t xml:space="preserve">POS17 F1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C19" t="inlineStr">
+      <x:c r="C19" t="inlineStr" s="45">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="D19" t="inlineStr">
+      <x:c r="D19" t="inlineStr" s="45">
         <x:is>
           <x:t xml:space="preserve">+6 µL</x:t>
         </x:is>
       </x:c>
-      <x:c r="E19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14 × 空白对照数量 + 6（质控类型为B的样本数）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F19" t="inlineStr">
+      <x:c r="E19" t="str" s="45">
+        <x:v>14 × B + 6 µL；B为空白对照数量，按SOP表9。</x:v>
+      </x:c>
+      <x:c r="F19" t="inlineStr" s="45">
         <x:is>
           <x:t xml:space="preserve">14 × B + 6</x:t>
         </x:is>
       </x:c>
-      <x:c r="G19" t="inlineStr">
+      <x:c r="G19" t="inlineStr" s="45">
         <x:is>
           <x:t xml:space="preserve">14 × B + 6</x:t>
         </x:is>
       </x:c>
-      <x:c r="H19" t="inlineStr">
+      <x:c r="H19" t="inlineStr" s="45">
         <x:is>
           <x:t xml:space="preserve">14 × B + 6</x:t>
         </x:is>
       </x:c>
-      <x:c r="I19" t="inlineStr">
+      <x:c r="I19" t="inlineStr" s="45">
         <x:is>
           <x:t xml:space="preserve">14 × B + 6</x:t>
         </x:is>
       </x:c>
-      <x:c r="J19" t="inlineStr">
+      <x:c r="J19" t="inlineStr" s="45">
         <x:is>
           <x:t xml:space="preserve">14 × B + 6</x:t>
         </x:is>
       </x:c>
-      <x:c r="K19" t="inlineStr">
+      <x:c r="K19" t="inlineStr" s="45">
         <x:is>
           <x:t xml:space="preserve">14 × B + 6</x:t>
         </x:is>
@@ -1476,23 +1457,21 @@
         <x:v>48</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="15" customHeight="1">
-      <x:c r="A4" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T1 cDNA引物</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="4" t="inlineStr">
+    <x:row r="4" ht="40" customHeight="1">
+      <x:c r="A4" s="46" t="str">
+        <x:v>T1 cDNA合成引物</x:v>
+      </x:c>
+      <x:c r="B4" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C1R1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C4" s="4" t="inlineStr">
+      <x:c r="C4" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="D4" s="4" t="inlineStr">
+      <x:c r="D4" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2 × N</x:t>
         </x:is>
@@ -1516,23 +1495,21 @@
         <x:v>96</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="45" customHeight="1">
-      <x:c r="A5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T2 cDNA缓冲液</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="4" t="inlineStr">
+    <x:row r="5" ht="40" customHeight="1">
+      <x:c r="A5" s="46" t="str">
+        <x:v>T2 一链合成缓冲液</x:v>
+      </x:c>
+      <x:c r="B5" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C2R1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C5" s="4" t="inlineStr">
+      <x:c r="C5" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="D5" s="4" t="inlineStr">
+      <x:c r="D5" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">第9列反应液总量 / 2；&gt;16通量增加2个完整POS7中转孔上游冗余</x:t>
         </x:is>
@@ -1556,23 +1533,21 @@
         <x:v>227.5</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="45" customHeight="1">
-      <x:c r="A6" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T3 cDNA酶</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" s="4" t="inlineStr">
+    <x:row r="6" ht="40" customHeight="1">
+      <x:c r="A6" s="46" t="str">
+        <x:v>T3 一链合成酶</x:v>
+      </x:c>
+      <x:c r="B6" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C3R1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C6" s="4" t="inlineStr">
+      <x:c r="C6" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="D6" s="4" t="inlineStr">
+      <x:c r="D6" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">第9列反应液总量 / 2；&gt;16通量增加2个完整POS7中转孔上游冗余</x:t>
         </x:is>
@@ -1596,23 +1571,19 @@
         <x:v>227.5</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="45" customHeight="1">
-      <x:c r="A7" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T4 TA缓冲液</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B7" s="4" t="inlineStr">
+    <x:row r="7" ht="40" customHeight="1">
+      <x:c r="A7" s="46" t="str">
+        <x:v>T4 靶向扩增缓冲液</x:v>
+      </x:c>
+      <x:c r="B7" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C1R2</x:t>
         </x:is>
       </x:c>
-      <x:c r="C7" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2 mL管</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D7" s="4" t="inlineStr">
+      <x:c r="C7" s="46" t="str">
+        <x:v>2.0 mL冻存管</x:v>
+      </x:c>
+      <x:c r="D7" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">第10列反应液总量 × 5/15；&gt;16通量增加2个完整POS7中转孔上游冗余</x:t>
         </x:is>
@@ -1636,23 +1607,21 @@
         <x:v>375</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="45" customHeight="1">
-      <x:c r="A8" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T5 TA酶</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B8" s="4" t="inlineStr">
+    <x:row r="8" ht="40" customHeight="1">
+      <x:c r="A8" s="46" t="str">
+        <x:v>T5 靶向扩增酶</x:v>
+      </x:c>
+      <x:c r="B8" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C2R2</x:t>
         </x:is>
       </x:c>
-      <x:c r="C8" s="4" t="inlineStr">
+      <x:c r="C8" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="D8" s="4" t="inlineStr">
+      <x:c r="D8" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">第10列反应液总量 × 3/15；&gt;16通量增加2个完整POS7中转孔上游冗余</x:t>
         </x:is>
@@ -1676,23 +1645,21 @@
         <x:v>225</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="45" customHeight="1">
-      <x:c r="A9" s="4" t="inlineStr">
+    <x:row r="9" ht="40" customHeight="1">
+      <x:c r="A9" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">T8 UDG酶</x:t>
         </x:is>
       </x:c>
-      <x:c r="B9" s="4" t="inlineStr">
+      <x:c r="B9" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C2R3</x:t>
         </x:is>
       </x:c>
-      <x:c r="C9" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2 mL管（手工预置C2R3）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D9" s="4" t="inlineStr">
+      <x:c r="C9" s="46" t="str">
+        <x:v>2.0 mL冻存管</x:v>
+      </x:c>
+      <x:c r="D9" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">第11列反应液总量 × 1/30；总量&gt;1421 µL时T8留在C2R3</x:t>
         </x:is>
@@ -1716,23 +1683,19 @@
         <x:v>67.67</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="45" customHeight="1">
-      <x:c r="A10" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T7 LA/PCR Mix</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B10" s="4" t="inlineStr">
+    <x:row r="10" ht="40" customHeight="1">
+      <x:c r="A10" s="46" t="str">
+        <x:v>T7 PCR Mix</x:v>
+      </x:c>
+      <x:c r="B10" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C1R3</x:t>
         </x:is>
       </x:c>
-      <x:c r="C10" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2 mL管</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D10" s="4" t="inlineStr">
+      <x:c r="C10" s="46" t="str">
+        <x:v>2.0 mL冻存管</x:v>
+      </x:c>
+      <x:c r="D10" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">第11列反应液总量 × 20/30；总量&gt;1421 µL时C2R3只配置T7+T8</x:t>
         </x:is>
@@ -1756,23 +1719,19 @@
         <x:v>1353.33</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="45" customHeight="1">
-      <x:c r="A11" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T2缓冲液总量</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B11" s="4" t="inlineStr">
+    <x:row r="11" ht="40" customHeight="1">
+      <x:c r="A11" s="46" t="str">
+        <x:v>T2溶解液（建库阶段代码消耗）</x:v>
+      </x:c>
+      <x:c r="B11" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS24 C1R2</x:t>
         </x:is>
       </x:c>
-      <x:c r="C11" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">8 mL管</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D11" s="4" t="inlineStr">
+      <x:c r="C11" s="46" t="str">
+        <x:v>8.0 mL冻存管</x:v>
+      </x:c>
+      <x:c r="D11" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">仅建库阶段：TA T2 + POS7 Col7 T2 + LA/PCR T2；G99 pooling预算另计入试剂分装表</x:t>
         </x:is>
@@ -1796,23 +1755,19 @@
         <x:v>4359.6</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="30" customHeight="1">
-      <x:c r="A12" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">磁珠总量</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B12" s="4" t="inlineStr">
+    <x:row r="12" ht="40" customHeight="1">
+      <x:c r="A12" s="46" t="str">
+        <x:v>T1磁珠</x:v>
+      </x:c>
+      <x:c r="B12" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS24 C1R1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C12" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">8 mL管</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D12" s="4" t="inlineStr">
+      <x:c r="C12" s="46" t="str">
+        <x:v>8.0 mL冻存管</x:v>
+      </x:c>
+      <x:c r="D12" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">TA磁珠 50 × 1.4 × N + LA磁珠 55 × N</x:t>
         </x:is>
@@ -1836,23 +1791,21 @@
         <x:v>6000</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="30" customHeight="1">
-      <x:c r="A13" s="4" t="inlineStr">
+    <x:row r="13" ht="40" customHeight="1">
+      <x:c r="A13" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">矿物油</x:t>
         </x:is>
       </x:c>
-      <x:c r="B13" s="4" t="inlineStr">
+      <x:c r="B13" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS24 C3R1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C13" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">8 mL管</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D13" s="4" t="inlineStr">
+      <x:c r="C13" s="46" t="str">
+        <x:v>8.0 mL冻存管</x:v>
+      </x:c>
+      <x:c r="D13" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">按当前代码逻辑计算矿物油预分装总量</x:t>
         </x:is>
@@ -1876,23 +1829,21 @@
         <x:v>2880</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="15" customHeight="1">
-      <x:c r="A14" s="4" t="inlineStr">
+    <x:row r="14" ht="40" customHeight="1">
+      <x:c r="A14" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">80%乙醇</x:t>
         </x:is>
       </x:c>
-      <x:c r="B14" s="4" t="inlineStr">
+      <x:c r="B14" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS3 reservoir</x:t>
         </x:is>
       </x:c>
-      <x:c r="C14" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">50 mL储液槽</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D14" s="4" t="inlineStr">
+      <x:c r="C14" s="46" t="str">
+        <x:v>50 mL试剂槽</x:v>
+      </x:c>
+      <x:c r="D14" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">195 × 5 × N</x:t>
         </x:is>
@@ -1916,21 +1867,19 @@
         <x:v>46800</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="15" customHeight="1">
-      <x:c r="A15" s="4" t="str">
-        <x:v>Qubit染液（G99/200/2000）</x:v>
-      </x:c>
-      <x:c r="B15" s="4" t="inlineStr">
+    <x:row r="15" ht="60" customHeight="1">
+      <x:c r="A15" s="46" t="str">
+        <x:v>Qubit染液（G99、200、2000全流程，前处理建库）</x:v>
+      </x:c>
+      <x:c r="B15" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS4 C1R1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C15" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">50 mL储液槽</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D15" s="4" t="inlineStr">
+      <x:c r="C15" s="46" t="str">
+        <x:v>50 mL避光试剂槽</x:v>
+      </x:c>
+      <x:c r="D15" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">单轮定量：217.8 × N</x:t>
         </x:is>
@@ -1960,17 +1909,17 @@
         <x:v>10454.400000000001</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="35.75" customHeight="1">
-      <x:c r="A16" t="str">
-        <x:v>Qubit染液（E25全流程）</x:v>
-      </x:c>
-      <x:c r="B16" t="str">
+    <x:row r="16" ht="60" customHeight="1">
+      <x:c r="A16" t="str" s="45">
+        <x:v>Qubit染液（E25全流程，前处理建库）</x:v>
+      </x:c>
+      <x:c r="B16" t="str" s="45">
         <x:v>POS4 C1R1</x:v>
       </x:c>
-      <x:c r="C16" t="str">
-        <x:v>50 mL储液槽</x:v>
-      </x:c>
-      <x:c r="D16" t="str">
+      <x:c r="C16" t="str" s="45">
+        <x:v>50 mL避光试剂槽</x:v>
+      </x:c>
+      <x:c r="D16" t="str" s="45">
         <x:v>两轮定量：2 × 217.8 × N</x:v>
       </x:c>
       <x:c r="E16" t="n">
@@ -1989,20 +1938,24 @@
         <x:f>H$3*217.8*2</x:f>
         <x:v>13939.2</x:v>
       </x:c>
-      <x:c r="I16"/>
-      <x:c r="J16"/>
-    </x:row>
-    <x:row r="17" ht="35.75" customHeight="1">
-      <x:c r="A17" t="str">
+      <x:c r="I16" t="str">
+        <x:v>/</x:v>
+      </x:c>
+      <x:c r="J16" t="str">
+        <x:v>/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="40" customHeight="1">
+      <x:c r="A17" t="str" s="45">
         <x:v>无核酸酶水（E25全流程）</x:v>
       </x:c>
-      <x:c r="B17" t="str">
+      <x:c r="B17" t="str" s="45">
         <x:v>POS24 A2</x:v>
       </x:c>
-      <x:c r="C17" t="str">
-        <x:v>8 mL管</x:v>
-      </x:c>
-      <x:c r="D17" t="str">
+      <x:c r="C17" t="str" s="45">
+        <x:v>8.0 mL冻存管</x:v>
+      </x:c>
+      <x:c r="D17" t="str" s="45">
         <x:v>最大代码消耗：27 × N</x:v>
       </x:c>
       <x:c r="E17" t="n">
@@ -2021,26 +1974,30 @@
         <x:f>H$3*27</x:f>
         <x:v>864</x:v>
       </x:c>
-      <x:c r="I17"/>
-      <x:c r="J17"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" t="inlineStr">
+      <x:c r="I17" t="str">
+        <x:v>/</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="40" customHeight="1">
+      <x:c r="A18" t="inlineStr" s="45">
         <x:is>
           <x:t xml:space="preserve">T12 空白对照</x:t>
         </x:is>
       </x:c>
-      <x:c r="B18" t="inlineStr">
+      <x:c r="B18" t="inlineStr" s="45">
         <x:is>
           <x:t xml:space="preserve">POS17 F1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C18" t="inlineStr">
+      <x:c r="C18" t="inlineStr" s="45">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="D18" t="inlineStr">
+      <x:c r="D18" t="inlineStr" s="45">
         <x:is>
           <x:t xml:space="preserve">14 × 空白对照数量（质控类型为B的样本数）</x:t>
         </x:is>
@@ -3240,10 +3197,8 @@
           <x:t xml:space="preserve">提取产物均一化</x:t>
         </x:is>
       </x:c>
-      <x:c r="C52" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">无核酸水最大代码消耗</x:t>
-        </x:is>
+      <x:c r="C52" t="str">
+        <x:v>无核酸酶水分装量（含冗余）</x:v>
       </x:c>
       <x:c r="D52" s="28" t="n">
         <x:f>CEILING(A52*27+320,10)</x:f>
@@ -3262,10 +3217,8 @@
           <x:t xml:space="preserve">提取产物均一化</x:t>
         </x:is>
       </x:c>
-      <x:c r="C53" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">无核酸水最大代码消耗</x:t>
-        </x:is>
+      <x:c r="C53" t="str">
+        <x:v>无核酸酶水分装量（含冗余）</x:v>
       </x:c>
       <x:c r="D53" s="28" t="n">
         <x:f>CEILING(A53*27+320,10)</x:f>
@@ -3284,10 +3237,8 @@
           <x:t xml:space="preserve">提取产物均一化</x:t>
         </x:is>
       </x:c>
-      <x:c r="C54" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">无核酸水最大代码消耗</x:t>
-        </x:is>
+      <x:c r="C54" t="str">
+        <x:v>无核酸酶水分装量（含冗余）</x:v>
       </x:c>
       <x:c r="D54" s="28" t="n">
         <x:f>CEILING(A54*27+320,10)</x:f>
@@ -3306,10 +3257,8 @@
           <x:t xml:space="preserve">提取产物均一化</x:t>
         </x:is>
       </x:c>
-      <x:c r="C55" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">无核酸水最大代码消耗</x:t>
-        </x:is>
+      <x:c r="C55" t="str">
+        <x:v>无核酸酶水分装量（含冗余）</x:v>
       </x:c>
       <x:c r="D55" s="28" t="n">
         <x:f>CEILING(A55*27+320,10)</x:f>
@@ -3328,10 +3277,8 @@
           <x:t xml:space="preserve">提取产物均一化</x:t>
         </x:is>
       </x:c>
-      <x:c r="C56" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">无核酸水最大代码消耗</x:t>
-        </x:is>
+      <x:c r="C56" t="str">
+        <x:v>无核酸酶水分装量（含冗余）</x:v>
       </x:c>
       <x:c r="D56" s="28" t="str">
         <x:v>不适用</x:v>
@@ -3349,10 +3296,8 @@
           <x:t xml:space="preserve">提取产物均一化</x:t>
         </x:is>
       </x:c>
-      <x:c r="C57" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">无核酸水最大代码消耗</x:t>
-        </x:is>
+      <x:c r="C57" t="str">
+        <x:v>无核酸酶水分装量（含冗余）</x:v>
       </x:c>
       <x:c r="D57" s="28" t="str">
         <x:v>不适用</x:v>
@@ -3608,14 +3553,14 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="4" ht="15" customHeight="1">
+    <x:row r="4" ht="85" customHeight="1">
       <x:c r="A4" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">范围</x:t>
         </x:is>
       </x:c>
-      <x:c r="B4" s="4" t="str">
-        <x:v>试剂分装主表覆盖 cDNA、TA、LA/PCR、两轮磁珠纯化、矿物油、乙醇和 Qubit 定量所需来源试剂；T2缓冲液额外包含G99 pooling预算。各测序平台makeDNB试剂见对应DNB试剂工作表。 E25全流程T2装量单列，覆盖非空白文库全8倍预稀释场景。</x:v>
+      <x:c r="B4" s="46" t="str">
+        <x:v>分装量、试剂名称、耗材和适用流程以当前SOP表9及表10-1/10-2/10-3为准；表内体积统一为µL（SOP中的mL已换算）。代码消耗及计算明细保留理论消耗和预算含义，不作为替代分装指令。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" customHeight="1">
@@ -3624,20 +3569,20 @@
           <x:t xml:space="preserve">分支规则</x:t>
         </x:is>
       </x:c>
-      <x:c r="B5" s="4" t="inlineStr">
+      <x:c r="B5" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">样本数≤16时，第9/10/11列反应液使用低通量P1直接分装；样本数&gt;16时使用POS7/P8中转。</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="6" ht="15" customHeight="1">
+    <x:row r="6" ht="85" customHeight="1">
       <x:c r="A6" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">来源死体积规则</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="4" t="str">
-        <x:v>0.5 mL管通常 +6 µL，T4和T5例外为 +10 µL；2 mL管 +15 µL；8 mL管通常 +320 µL；磁珠总量特例 +400 µL；50 mL试剂槽按实际管底余量配置，80%乙醇 +3200 µL，Qubit染液 +6510 µL。 T1 cDNA引物来源冗余为10 µL，分装量向上取整到10 µL。</x:v>
+      <x:c r="B6" s="46" t="str">
+        <x:v>来源冗余为计算下限，实际分装量以SOP取整后的数值为准：T1 +10 µL；T2/T3一链试剂 +6 µL；T4/T5 +10 µL；T7 +15 µL；8 mL管通常 +320 µL，磁珠 +400 µL；乙醇 +3200 µL，Qubit +6510 µL。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" customHeight="1">
@@ -3646,7 +3591,7 @@
           <x:t xml:space="preserve">POS7封顶曲线</x:t>
         </x:is>
       </x:c>
-      <x:c r="B7" s="4" t="inlineStr">
+      <x:c r="B7" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS7反应液中转孔仍按：活跃下游列数 × 单次吸取体积 + 20 µL总冗余；样本数&gt;16时，上游mixing tube另增加2个完整POS7中转孔的体积。</x:t>
         </x:is>
@@ -3658,42 +3603,40 @@
           <x:t xml:space="preserve">混合管死体积</x:t>
         </x:is>
       </x:c>
-      <x:c r="B8" s="4" t="inlineStr">
+      <x:c r="B8" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 Col4 Row1 cDNA混合管基础死体积15 µL；POS17 Col4 Row2 TA混合管25 µL；POS17 C2R3 LA/PCR混合管30 µL。样本数&gt;16时三者另加2个完整POS7中转孔上游冗余。</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="9" ht="15" customHeight="1">
+    <x:row r="9" ht="85" customHeight="1">
       <x:c r="A9" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">T2缓冲液共用来源</x:t>
         </x:is>
       </x:c>
-      <x:c r="B9" s="4" t="str">
-        <x:v>POS24 C1R2合并建库阶段TA、POS7 Col7中转和LA/PCR的T2消耗。其他路线保留原G99 pooling预算；E25全流程按N−1个非空白文库全8倍稀释、1个DNB计入35 µL/孔和动态补液上限。分装1500/2400/3600/5000 µL均已含320 µL来源冗余。提取均一化无核酸酶水为独立来源，不计入T2。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="15" customHeight="1">
+      <x:c r="B9" s="46" t="str">
+        <x:v>POS24 C1R2合并建库阶段TA、POS7 Col7中转和LA/PCR的T2消耗。其他路线保留原G99 pooling预算；E25全流程按N−1个非空白文库全8倍稀释、1个DNB计入35 µL/孔和动态补液上限。分装2100/3000/4200/5000 µL：各档计算预算先计入320 µL来源冗余，向上取整到100 µL，再统一增加600 µL额外备液。提取均一化无核酸酶水为独立来源，不计入T2。 上机前准备流程按SOP表10各配T2溶解液6000 µL；8 mL管用后回收，须盖黑色胶塞，全流程不重复加配。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="85" customHeight="1">
       <x:c r="A10" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">乙醇</x:t>
         </x:is>
       </x:c>
-      <x:c r="B10" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">POS3到POS7的乙醇预分装按每个活跃通道195 µL × 5轮计算，并额外加入50 mL储液槽余量。</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="15" customHeight="1">
+      <x:c r="B10" s="46" t="str">
+        <x:v>POS3乙醇分装按195 × 5 × N + 3200 µL，向上取1000 µL；8/16/24/32/40/48例为11000/19000/27000/35000/43000/50000 µL，与SOP表9一致。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="85" customHeight="1">
       <x:c r="A11" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Qubit染液</x:t>
         </x:is>
       </x:c>
-      <x:c r="B11" s="4" t="str">
-        <x:v>POS4 C1R1分装量：G99、200、2000全流程为217.8 × N + 6510 µL；E25全流程为2 × 217.8 × N + 6510 µL；均向上取1000 µL。</x:v>
+      <x:c r="B11" s="46" t="str">
+        <x:v>按SOP表9：G99、200、2000全流程，前处理建库为9000/10000/12000/14000/16000/17000 µL；E25全流程，前处理建库为10000/14000/17000/21000 µL（最多32例）。单轮/两轮用量分别加6510 µL，向上取1000 µL。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" customHeight="1">
@@ -3744,7 +3687,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="85" customHeight="1">
       <x:c r="A16" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">提取产物均一化</x:t>
@@ -3754,7 +3697,7 @@
         <x:v>E25全流程提取回收45 µL；取2.2 µL在POS14 Col7-10定量。目标20 ng/µL、30 µL；原始浓度低于20 ng/µL时不补水，直接转移30 µL。</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="85" customHeight="1">
       <x:c r="A17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">均一化范围</x:t>
@@ -3766,7 +3709,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="85" customHeight="1">
       <x:c r="A18" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">板位与枪头</x:t>
@@ -4149,7 +4092,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="13" ht="15" customHeight="1">
+    <x:row r="13" ht="35" customHeight="1">
       <x:c r="A13" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS8</x:t>
@@ -4175,7 +4118,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="14" ht="30" customHeight="1">
+    <x:row r="14" ht="35" customHeight="1">
       <x:c r="A14" s="12" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS8</x:t>
@@ -4201,7 +4144,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="15" ht="15" customHeight="1">
+    <x:row r="15" ht="35" customHeight="1">
       <x:c r="A15" s="12" t="str">
         <x:v>POS8</x:v>
       </x:c>
@@ -4223,7 +4166,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="16" ht="15" customHeight="1">
+    <x:row r="16" ht="35" customHeight="1">
       <x:c r="A16" s="12" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS14</x:t>
@@ -4241,7 +4184,7 @@
       <x:c r="E16" s="7" t="n"/>
       <x:c r="F16" s="7" t="n"/>
     </x:row>
-    <x:row r="17" ht="15" customHeight="1">
+    <x:row r="17" ht="35" customHeight="1">
       <x:c r="A17" s="12" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS14</x:t>
@@ -4259,7 +4202,7 @@
       <x:c r="E17" s="7" t="n"/>
       <x:c r="F17" s="7" t="n"/>
     </x:row>
-    <x:row r="18" ht="15" customHeight="1">
+    <x:row r="18" ht="35" customHeight="1">
       <x:c r="A18" s="15" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS24 A2</x:t>
@@ -4309,179 +4252,212 @@
       <x:c r="F1" s="31" t="n"/>
       <x:c r="G1" s="32" t="n"/>
     </x:row>
-    <x:row r="2" ht="15" customHeight="1">
-      <x:c r="A2" s="26" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">E25 full 与 sequencing prep 的 makeDNB 试剂位置和机器取液逻辑一致；Mix I 大体积加入 Mix II 小体积管。单位：µL。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" s="31" t="n"/>
-      <x:c r="C2" s="31" t="n"/>
-      <x:c r="D2" s="31" t="n"/>
-      <x:c r="E2" s="31" t="n"/>
-      <x:c r="F2" s="31" t="n"/>
-      <x:c r="G2" s="32" t="n"/>
-    </x:row>
-    <x:row r="3" ht="32" customHeight="1">
-      <x:c r="A3" s="18" t="inlineStr">
+    <x:row r="2" ht="55" customHeight="1">
+      <x:c r="A2" s="36" t="str">
+        <x:v>E25全流程每轮1个DNB；上机前准备最多3个DNB。按SOP表10-3分装，单位µL；T2仅上机前准备另配6000 µL，全流程用量见表9。</x:v>
+      </x:c>
+      <x:c r="B2" s="37" t="n"/>
+      <x:c r="C2" s="37" t="n"/>
+      <x:c r="D2" s="37" t="n"/>
+      <x:c r="E2" s="37" t="n"/>
+      <x:c r="F2" s="37" t="n"/>
+      <x:c r="G2" s="44" t="n"/>
+    </x:row>
+    <x:row r="3" ht="35" customHeight="1">
+      <x:c r="A3" s="38" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">试剂名称</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" s="18" t="inlineStr">
+      <x:c r="B3" s="38" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">耗材</x:t>
         </x:is>
       </x:c>
-      <x:c r="C3" s="18" t="inlineStr">
+      <x:c r="C3" s="38" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">台面位置</x:t>
         </x:is>
       </x:c>
-      <x:c r="D3" s="18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">配置公式</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E3" s="33" t="n">
+      <x:c r="D3" s="38" t="str">
+        <x:v>配置公式（D为DNB个数）</x:v>
+      </x:c>
+      <x:c r="E3" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F3" s="33" t="n">
+      <x:c r="F3" s="39" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="G3" s="33" t="n">
+      <x:c r="G3" s="39" t="n">
         <x:v>3</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="20" t="str">
-        <x:v>DNB制备缓冲液（SB）</x:v>
-      </x:c>
-      <x:c r="B4" s="20" t="inlineStr">
+    <x:row r="4" ht="45" customHeight="1">
+      <x:c r="A4" s="40" t="str">
+        <x:v>DNB制备缓冲液(OS-V2.0-SB)</x:v>
+      </x:c>
+      <x:c r="B4" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="C4" s="20" t="inlineStr">
+      <x:c r="C4" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C1R5</x:t>
         </x:is>
       </x:c>
-      <x:c r="D4" s="20" t="inlineStr">
+      <x:c r="D4" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">20 × D + 20</x:t>
         </x:is>
       </x:c>
-      <x:c r="E4" s="34" t="n">
+      <x:c r="E4" s="41" t="n">
         <x:f>20*E$3+20</x:f>
         <x:v>40</x:v>
       </x:c>
-      <x:c r="F4" s="34" t="n">
+      <x:c r="F4" s="41" t="n">
         <x:f>20*F$3+20</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="G4" s="34" t="n">
+      <x:c r="G4" s="41" t="n">
         <x:f>20*G$3+20</x:f>
         <x:v>80</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DNB聚合酶混合液 I（OS）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="20" t="inlineStr">
+    <x:row r="5" ht="45" customHeight="1">
+      <x:c r="A5" s="40" t="str">
+        <x:v>DNB聚合酶混合液Ⅰ(OS)</x:v>
+      </x:c>
+      <x:c r="B5" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="C5" s="20" t="inlineStr">
+      <x:c r="C5" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C2R5</x:t>
         </x:is>
       </x:c>
-      <x:c r="D5" s="20" t="str">
+      <x:c r="D5" s="40" t="str">
         <x:v>40×(D+0.5)+6，向上取10</x:v>
       </x:c>
-      <x:c r="E5" s="34" t="n">
+      <x:c r="E5" s="41" t="n">
         <x:f>CEILING(40*(E$3+0.5)+6,10)</x:f>
         <x:v>70</x:v>
       </x:c>
-      <x:c r="F5" s="34" t="n">
+      <x:c r="F5" s="41" t="n">
         <x:f>CEILING(40*(F$3+0.5)+6,10)</x:f>
         <x:v>110</x:v>
       </x:c>
-      <x:c r="G5" s="34" t="n">
+      <x:c r="G5" s="41" t="n">
         <x:f>CEILING(40*(G$3+0.5)+6,10)</x:f>
         <x:v>150</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="30" customHeight="1">
-      <x:c r="A6" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DNB聚合酶混合液 II（OS）†</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" s="20" t="inlineStr">
+    <x:row r="6" ht="45" customHeight="1">
+      <x:c r="A6" s="40" t="str">
+        <x:v>DNB聚合酶混合液Ⅱ（OS）</x:v>
+      </x:c>
+      <x:c r="B6" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="C6" s="20" t="inlineStr">
+      <x:c r="C6" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C3R5</x:t>
         </x:is>
       </x:c>
-      <x:c r="D6" s="20" t="str">
+      <x:c r="D6" s="40" t="str">
         <x:v>4 × (D + 0.5)</x:v>
       </x:c>
-      <x:c r="E6" s="34" t="n">
+      <x:c r="E6" s="41" t="n">
         <x:f>4*(E$3+0.5)</x:f>
         <x:v>6</x:v>
       </x:c>
-      <x:c r="F6" s="34" t="n">
+      <x:c r="F6" s="41" t="n">
         <x:f>4*(F$3+0.5)</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="G6" s="34" t="n">
+      <x:c r="G6" s="41" t="n">
         <x:f>4*(G$3+0.5)</x:f>
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="20" t="inlineStr">
+    <x:row r="7" ht="45" customHeight="1">
+      <x:c r="A7" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DNB终止缓冲液</x:t>
         </x:is>
       </x:c>
-      <x:c r="B7" s="20" t="inlineStr">
+      <x:c r="B7" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="C7" s="20" t="inlineStr">
+      <x:c r="C7" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C4R5</x:t>
         </x:is>
       </x:c>
-      <x:c r="D7" s="20" t="inlineStr">
+      <x:c r="D7" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">20 × D + 20</x:t>
         </x:is>
       </x:c>
-      <x:c r="E7" s="34" t="n">
+      <x:c r="E7" s="41" t="n">
         <x:f>20*E$3+20</x:f>
         <x:v>40</x:v>
       </x:c>
-      <x:c r="F7" s="34" t="n">
+      <x:c r="F7" s="41" t="n">
         <x:f>20*F$3+20</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="G7" s="34" t="n">
+      <x:c r="G7" s="41" t="n">
         <x:f>20*G$3+20</x:f>
         <x:v>80</x:v>
       </x:c>
+    </x:row>
+    <x:row r="8" ht="85" customHeight="1">
+      <x:c r="A8" s="40" t="str">
+        <x:v>T2溶解液</x:v>
+      </x:c>
+      <x:c r="B8" s="40" t="str">
+        <x:v>8 mL管（用后回收，须盖黑色胶塞）</x:v>
+      </x:c>
+      <x:c r="C8" s="40" t="str">
+        <x:v>POS24 C1R2</x:v>
+      </x:c>
+      <x:c r="D8" s="40" t="str">
+        <x:v>仅上机前准备需配；全流程见SOP表9</x:v>
+      </x:c>
+      <x:c r="E8" s="41" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="F8" s="41" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="G8" s="41" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="45"/>
+      <x:c r="B9" s="45"/>
+      <x:c r="C9" s="45"/>
+      <x:c r="D9" s="45"/>
+      <x:c r="E9" s="45"/>
+      <x:c r="F9" s="45"/>
+      <x:c r="G9" s="45"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="45"/>
+      <x:c r="B10" s="45"/>
+      <x:c r="C10" s="45"/>
+      <x:c r="D10" s="45"/>
+      <x:c r="E10" s="45"/>
+      <x:c r="F10" s="45"/>
+      <x:c r="G10" s="45"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4519,336 +4495,279 @@
       <x:c r="I1" s="31" t="n"/>
       <x:c r="J1" s="32" t="n"/>
     </x:row>
-    <x:row r="2" ht="15" customHeight="1">
-      <x:c r="A2" s="26" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">G99 full 与 sequencing prep 的 makeDNB 试剂位置和机器取液逻辑一致；D1加入D2，Mix I加入Mix II。D1按整µL向上取整。单位：µL。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" s="31" t="n"/>
-      <x:c r="C2" s="31" t="n"/>
-      <x:c r="D2" s="31" t="n"/>
-      <x:c r="E2" s="31" t="n"/>
-      <x:c r="F2" s="31" t="n"/>
-      <x:c r="G2" s="31" t="n"/>
+    <x:row r="2" ht="55" customHeight="1">
+      <x:c r="A2" s="36" t="str">
+        <x:v>G99全流程每轮1个DNB；上机前准备最多3个DNB。按SOP表10-2分装，单位µL；T2仅上机前准备另配6000 µL，全流程用量见表9。</x:v>
+      </x:c>
+      <x:c r="B2" s="37" t="n"/>
+      <x:c r="C2" s="37" t="n"/>
+      <x:c r="D2" s="37" t="n"/>
+      <x:c r="E2" s="37" t="n"/>
+      <x:c r="F2" s="37" t="n"/>
+      <x:c r="G2" s="37" t="n"/>
       <x:c r="H2" s="31" t="n"/>
       <x:c r="I2" s="31" t="n"/>
       <x:c r="J2" s="32" t="n"/>
     </x:row>
-    <x:row r="3" ht="32" customHeight="1">
-      <x:c r="A3" s="18" t="inlineStr">
+    <x:row r="3" ht="35" customHeight="1">
+      <x:c r="A3" s="38" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">试剂名称</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" s="18" t="inlineStr">
+      <x:c r="B3" s="38" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">耗材</x:t>
         </x:is>
       </x:c>
-      <x:c r="C3" s="18" t="inlineStr">
+      <x:c r="C3" s="38" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">台面位置</x:t>
         </x:is>
       </x:c>
-      <x:c r="D3" s="18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">配置公式</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E3" s="33" t="n">
+      <x:c r="D3" s="38" t="str">
+        <x:v>配置公式（D为DNB个数）</x:v>
+      </x:c>
+      <x:c r="E3" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F3" s="33" t="n">
+      <x:c r="F3" s="39" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="G3" s="33" t="n">
+      <x:c r="G3" s="39" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H3" s="33" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="I3" s="33" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="J3" s="33" t="n">
-        <x:v>6</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">环化反应缓冲液（D1）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="20" t="inlineStr">
+      <x:c r="H3" s="33"/>
+      <x:c r="I3" s="33"/>
+      <x:c r="J3" s="33"/>
+    </x:row>
+    <x:row r="4" ht="45" customHeight="1">
+      <x:c r="A4" s="40" t="str">
+        <x:v>环化反应缓冲液</x:v>
+      </x:c>
+      <x:c r="B4" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="C4" s="20" t="inlineStr">
+      <x:c r="C4" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C1R4</x:t>
         </x:is>
       </x:c>
-      <x:c r="D4" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">ROUNDUP[11.6 × (D + 1) + 6]</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" s="34" t="n">
-        <x:f>ROUNDUP(11.6*(E$3+1)+6,0)</x:f>
+      <x:c r="D4" s="40" t="str">
+        <x:v>11.6 × (D + 1) + 6，向上取10</x:v>
+      </x:c>
+      <x:c r="E4" s="41" t="n">
+        <x:f>CEILING(11.6*(E$3+1)+6,10)</x:f>
         <x:v>30</x:v>
       </x:c>
-      <x:c r="F4" s="34" t="n">
-        <x:f>ROUNDUP(11.6*(F$3+1)+6,0)</x:f>
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="G4" s="34" t="n">
-        <x:f>ROUNDUP(11.6*(G$3+1)+6,0)</x:f>
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="H4" s="34" t="n">
-        <x:f>ROUNDUP(11.6*(H$3+1)+6,0)</x:f>
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="I4" s="34" t="n">
-        <x:f>ROUNDUP(11.6*(I$3+1)+6,0)</x:f>
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="J4" s="34" t="n">
-        <x:f>ROUNDUP(11.6*(J$3+1)+6,0)</x:f>
-        <x:v>88</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">环化反应酶（D2）†</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="20" t="inlineStr">
+      <x:c r="F4" s="41" t="n">
+        <x:f>CEILING(11.6*(F$3+1)+6,10)</x:f>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="G4" s="41" t="n">
+        <x:f>CEILING(11.6*(G$3+1)+6,10)</x:f>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="H4" s="34"/>
+      <x:c r="I4" s="34"/>
+      <x:c r="J4" s="34"/>
+    </x:row>
+    <x:row r="5" ht="45" customHeight="1">
+      <x:c r="A5" s="40" t="str">
+        <x:v>连接酶</x:v>
+      </x:c>
+      <x:c r="B5" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="C5" s="20" t="inlineStr">
+      <x:c r="C5" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C2R4</x:t>
         </x:is>
       </x:c>
-      <x:c r="D5" s="20" t="inlineStr">
+      <x:c r="D5" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 × (D + 1)</x:t>
         </x:is>
       </x:c>
-      <x:c r="E5" s="34" t="n">
+      <x:c r="E5" s="41" t="n">
         <x:f>0.5*(E$3+1)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F5" s="34" t="n">
+      <x:c r="F5" s="41" t="n">
         <x:f>0.5*(F$3+1)</x:f>
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="G5" s="34" t="n">
+      <x:c r="G5" s="41" t="n">
         <x:f>0.5*(G$3+1)</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H5" s="34" t="n">
-        <x:f>0.5*(H$3+1)</x:f>
-        <x:v>2.5</x:v>
-      </x:c>
-      <x:c r="I5" s="34" t="n">
-        <x:f>0.5*(I$3+1)</x:f>
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="J5" s="34" t="n">
-        <x:f>0.5*(J$3+1)</x:f>
-        <x:v>3.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="30" customHeight="1">
-      <x:c r="A6" s="20" t="inlineStr">
+      <x:c r="H5" s="34"/>
+      <x:c r="I5" s="34"/>
+      <x:c r="J5" s="34"/>
+    </x:row>
+    <x:row r="6" ht="45" customHeight="1">
+      <x:c r="A6" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DNB制备缓冲液（SB）</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="20" t="inlineStr">
+      <x:c r="B6" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="C6" s="20" t="inlineStr">
+      <x:c r="C6" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C3R5</x:t>
         </x:is>
       </x:c>
-      <x:c r="D6" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14 × D + 6</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E6" s="34" t="n">
-        <x:f>14*E$3+6</x:f>
+      <x:c r="D6" s="40" t="str">
+        <x:v>14 × D + 6，向上取10</x:v>
+      </x:c>
+      <x:c r="E6" s="41" t="n">
+        <x:f>CEILING(14*E$3+6,10)</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="F6" s="34" t="n">
-        <x:f>14*F$3+6</x:f>
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="G6" s="34" t="n">
-        <x:f>14*G$3+6</x:f>
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="H6" s="34" t="n">
-        <x:f>14*H$3+6</x:f>
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="I6" s="34" t="n">
-        <x:f>14*I$3+6</x:f>
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="J6" s="34" t="n">
-        <x:f>14*J$3+6</x:f>
-        <x:v>90</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">聚合酶 Mix I（E1）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B7" s="20" t="inlineStr">
+      <x:c r="F6" s="41" t="n">
+        <x:f>CEILING(14*F$3+6,10)</x:f>
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G6" s="41" t="n">
+        <x:f>CEILING(14*G$3+6,10)</x:f>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="H6" s="34"/>
+      <x:c r="I6" s="34"/>
+      <x:c r="J6" s="34"/>
+    </x:row>
+    <x:row r="7" ht="45" customHeight="1">
+      <x:c r="A7" s="40" t="str">
+        <x:v>DNB聚合酶混合液Ⅰ</x:v>
+      </x:c>
+      <x:c r="B7" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="C7" s="20" t="inlineStr">
+      <x:c r="C7" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C1R5</x:t>
         </x:is>
       </x:c>
-      <x:c r="D7" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">20 × (D + 0.5) + 6</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E7" s="34" t="n">
-        <x:f>20*(E$3+0.5)+6</x:f>
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F7" s="34" t="n">
-        <x:f>20*(F$3+0.5)+6</x:f>
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="G7" s="34" t="n">
-        <x:f>20*(G$3+0.5)+6</x:f>
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="H7" s="34" t="n">
-        <x:f>20*(H$3+0.5)+6</x:f>
-        <x:v>96</x:v>
-      </x:c>
-      <x:c r="I7" s="34" t="n">
-        <x:f>20*(I$3+0.5)+6</x:f>
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="J7" s="34" t="n">
-        <x:f>20*(J$3+0.5)+6</x:f>
-        <x:v>136</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="30" customHeight="1">
-      <x:c r="A8" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">聚合酶 Mix II（E2）†</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B8" s="20" t="inlineStr">
+      <x:c r="D7" s="40" t="str">
+        <x:v>20 × (D + 0.5) + 6，向上取10</x:v>
+      </x:c>
+      <x:c r="E7" s="41" t="n">
+        <x:f>CEILING(20*(E$3+0.5)+6,10)</x:f>
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F7" s="41" t="n">
+        <x:f>CEILING(20*(F$3+0.5)+6,10)</x:f>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G7" s="41" t="n">
+        <x:f>CEILING(20*(G$3+0.5)+6,10)</x:f>
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="H7" s="34"/>
+      <x:c r="I7" s="34"/>
+      <x:c r="J7" s="34"/>
+    </x:row>
+    <x:row r="8" ht="45" customHeight="1">
+      <x:c r="A8" s="40" t="str">
+        <x:v>DNB聚合酶混合液Ⅱ（LC）</x:v>
+      </x:c>
+      <x:c r="B8" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="C8" s="20" t="inlineStr">
+      <x:c r="C8" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C2R5</x:t>
         </x:is>
       </x:c>
-      <x:c r="D8" s="20" t="inlineStr">
+      <x:c r="D8" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2 × (D + 0.5)</x:t>
         </x:is>
       </x:c>
-      <x:c r="E8" s="34" t="n">
+      <x:c r="E8" s="41" t="n">
         <x:f>2*(E$3+0.5)</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="F8" s="34" t="n">
+      <x:c r="F8" s="41" t="n">
         <x:f>2*(F$3+0.5)</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G8" s="34" t="n">
+      <x:c r="G8" s="41" t="n">
         <x:f>2*(G$3+0.5)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="H8" s="34" t="n">
-        <x:f>2*(H$3+0.5)</x:f>
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="I8" s="34" t="n">
-        <x:f>2*(I$3+0.5)</x:f>
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="J8" s="34" t="n">
-        <x:f>2*(J$3+0.5)</x:f>
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="30" customHeight="1">
-      <x:c r="A9" s="20" t="inlineStr">
+      <x:c r="H8" s="34"/>
+      <x:c r="I8" s="34"/>
+      <x:c r="J8" s="34"/>
+    </x:row>
+    <x:row r="9" ht="45" customHeight="1">
+      <x:c r="A9" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DNB终止缓冲液</x:t>
         </x:is>
       </x:c>
-      <x:c r="B9" s="20" t="inlineStr">
+      <x:c r="B9" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.5 mL冻存管</x:t>
         </x:is>
       </x:c>
-      <x:c r="C9" s="20" t="inlineStr">
+      <x:c r="C9" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">POS17 C4R5</x:t>
         </x:is>
       </x:c>
-      <x:c r="D9" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14 × D + 6</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E9" s="34" t="n">
-        <x:f>14*E$3+6</x:f>
+      <x:c r="D9" s="40" t="str">
+        <x:v>14 × D + 6，向上取10</x:v>
+      </x:c>
+      <x:c r="E9" s="41" t="n">
+        <x:f>CEILING(14*E$3+6,10)</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="F9" s="34" t="n">
-        <x:f>14*F$3+6</x:f>
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="G9" s="34" t="n">
-        <x:f>14*G$3+6</x:f>
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="H9" s="34" t="n">
-        <x:f>14*H$3+6</x:f>
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="I9" s="34" t="n">
-        <x:f>14*I$3+6</x:f>
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="J9" s="34" t="n">
-        <x:f>14*J$3+6</x:f>
-        <x:v>90</x:v>
+      <x:c r="F9" s="41" t="n">
+        <x:f>CEILING(14*F$3+6,10)</x:f>
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G9" s="41" t="n">
+        <x:f>CEILING(14*G$3+6,10)</x:f>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="H9" s="34"/>
+      <x:c r="I9" s="34"/>
+      <x:c r="J9" s="34"/>
+    </x:row>
+    <x:row r="10" ht="85" customHeight="1">
+      <x:c r="A10" s="40" t="str">
+        <x:v>T2溶解液</x:v>
+      </x:c>
+      <x:c r="B10" s="40" t="str">
+        <x:v>8 mL管（用后回收，须盖黑色胶塞）</x:v>
+      </x:c>
+      <x:c r="C10" s="40" t="str">
+        <x:v>POS24 C1R2</x:v>
+      </x:c>
+      <x:c r="D10" s="40" t="str">
+        <x:v>仅上机前准备需配；全流程见SOP表9</x:v>
+      </x:c>
+      <x:c r="E10" s="41" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="F10" s="41" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="G10" s="41" t="n">
+        <x:v>6000</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4883,195 +4802,208 @@
       <x:c r="G1" s="31" t="n"/>
       <x:c r="H1" s="32" t="n"/>
     </x:row>
-    <x:row r="2" ht="15" customHeight="1">
-      <x:c r="A2" s="26" t="str">
-        <x:v>MGISEQ-200/2000全流程每轮仅配置1个DNB；上机前准备按实际DNB个数配置，最多3个DNB。下表与SOP表10-1一致，按实际DNB个数选择分装量。单位：µL。</x:v>
-      </x:c>
-      <x:c r="B2" s="31" t="n"/>
-      <x:c r="C2" s="31" t="n"/>
-      <x:c r="D2" s="31" t="n"/>
-      <x:c r="E2" s="31" t="n"/>
-      <x:c r="F2" s="31" t="n"/>
-      <x:c r="G2" s="31" t="n"/>
+    <x:row r="2" ht="55" customHeight="1">
+      <x:c r="A2" s="36" t="str">
+        <x:v>MGISEQ-200/2000全流程每轮1个DNB；上机前准备最多3个DNB。按SOP表10-1分装，单位µL；T2仅上机前准备另配6000 µL，全流程用量见表9。</x:v>
+      </x:c>
+      <x:c r="B2" s="37" t="n"/>
+      <x:c r="C2" s="37" t="n"/>
+      <x:c r="D2" s="37" t="n"/>
+      <x:c r="E2" s="37" t="n"/>
+      <x:c r="F2" s="37" t="n"/>
+      <x:c r="G2" s="37" t="n"/>
       <x:c r="H2" s="32" t="n"/>
     </x:row>
-    <x:row r="3" ht="32" customHeight="1">
-      <x:c r="A3" s="18" t="str">
+    <x:row r="3" ht="35" customHeight="1">
+      <x:c r="A3" s="38" t="str">
         <x:v>试剂名称</x:v>
       </x:c>
-      <x:c r="B3" s="18" t="str">
+      <x:c r="B3" s="38" t="str">
         <x:v>耗材</x:v>
       </x:c>
-      <x:c r="C3" s="18" t="str">
+      <x:c r="C3" s="38" t="str">
         <x:v>台面位置</x:v>
       </x:c>
-      <x:c r="D3" s="18" t="str">
+      <x:c r="D3" s="38" t="str">
         <x:v>分装口径</x:v>
       </x:c>
-      <x:c r="E3" s="18" t="str">
+      <x:c r="E3" s="38" t="str">
         <x:v>DNB-1个</x:v>
       </x:c>
-      <x:c r="F3" s="18" t="str">
+      <x:c r="F3" s="38" t="str">
         <x:v>DNB-2个</x:v>
       </x:c>
-      <x:c r="G3" s="18" t="str">
+      <x:c r="G3" s="38" t="str">
         <x:v>DNB-3个</x:v>
       </x:c>
       <x:c r="H3" s="18"/>
     </x:row>
-    <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="22" t="str">
-        <x:v>环化反应缓冲液（D1）</x:v>
-      </x:c>
-      <x:c r="B4" s="22" t="str">
+    <x:row r="4" ht="45" customHeight="1">
+      <x:c r="A4" s="42" t="str">
+        <x:v>环化反应缓冲液</x:v>
+      </x:c>
+      <x:c r="B4" s="42" t="str">
         <x:v>0.5 mL冻存管</x:v>
       </x:c>
-      <x:c r="C4" s="22" t="str">
+      <x:c r="C4" s="42" t="str">
         <x:v>POS17 C1R4</x:v>
       </x:c>
-      <x:c r="D4" s="22" t="str">
+      <x:c r="D4" s="42" t="str">
         <x:v>按SOP表10-1</x:v>
       </x:c>
-      <x:c r="E4" s="35" t="n">
+      <x:c r="E4" s="43" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="F4" s="35" t="n">
+      <x:c r="F4" s="43" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="G4" s="35" t="n">
+      <x:c r="G4" s="43" t="n">
         <x:v>60</x:v>
       </x:c>
       <x:c r="H4" s="35"/>
     </x:row>
-    <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="20" t="str">
-        <x:v>环化反应酶（D2）†</x:v>
-      </x:c>
-      <x:c r="B5" s="20" t="str">
+    <x:row r="5" ht="45" customHeight="1">
+      <x:c r="A5" s="40" t="str">
+        <x:v>连接酶</x:v>
+      </x:c>
+      <x:c r="B5" s="40" t="str">
         <x:v>0.5 mL冻存管</x:v>
       </x:c>
-      <x:c r="C5" s="20" t="str">
+      <x:c r="C5" s="40" t="str">
         <x:v>POS17 C2R4</x:v>
       </x:c>
-      <x:c r="D5" s="20" t="str">
+      <x:c r="D5" s="40" t="str">
         <x:v>按SOP表10-1手工分装</x:v>
       </x:c>
-      <x:c r="E5" s="34" t="n">
+      <x:c r="E5" s="41" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F5" s="34" t="n">
+      <x:c r="F5" s="41" t="n">
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="G5" s="34" t="n">
+      <x:c r="G5" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="H5" s="34"/>
     </x:row>
-    <x:row r="6" ht="30" customHeight="1">
-      <x:c r="A6" s="20" t="str">
-        <x:v>DNB制备缓冲液（SB）</x:v>
-      </x:c>
-      <x:c r="B6" s="20" t="str">
+    <x:row r="6" ht="45" customHeight="1">
+      <x:c r="A6" s="40" t="str">
+        <x:v>DNB制备缓冲液</x:v>
+      </x:c>
+      <x:c r="B6" s="40" t="str">
         <x:v>0.5 mL冻存管</x:v>
       </x:c>
-      <x:c r="C6" s="20" t="str">
+      <x:c r="C6" s="40" t="str">
         <x:v>POS17 C3R5</x:v>
       </x:c>
-      <x:c r="D6" s="20" t="str">
+      <x:c r="D6" s="40" t="str">
         <x:v>按SOP表10-1</x:v>
       </x:c>
-      <x:c r="E6" s="34" t="n">
+      <x:c r="E6" s="41" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="F6" s="34" t="n">
+      <x:c r="F6" s="41" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="G6" s="34" t="n">
+      <x:c r="G6" s="41" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="H6" s="34"/>
     </x:row>
-    <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="20" t="str">
-        <x:v>聚合酶 Mix I（E1）</x:v>
-      </x:c>
-      <x:c r="B7" s="20" t="str">
+    <x:row r="7" ht="45" customHeight="1">
+      <x:c r="A7" s="40" t="str">
+        <x:v>DNB聚合酶混合液Ⅰ</x:v>
+      </x:c>
+      <x:c r="B7" s="40" t="str">
         <x:v>0.5 mL冻存管</x:v>
       </x:c>
-      <x:c r="C7" s="20" t="str">
+      <x:c r="C7" s="40" t="str">
         <x:v>POS17 C1R5</x:v>
       </x:c>
-      <x:c r="D7" s="20" t="str">
+      <x:c r="D7" s="40" t="str">
         <x:v>按SOP表10-1</x:v>
       </x:c>
-      <x:c r="E7" s="34" t="n">
+      <x:c r="E7" s="41" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="F7" s="34" t="n">
+      <x:c r="F7" s="41" t="n">
         <x:v>110</x:v>
       </x:c>
-      <x:c r="G7" s="34" t="n">
+      <x:c r="G7" s="41" t="n">
         <x:v>150</x:v>
       </x:c>
       <x:c r="H7" s="34"/>
     </x:row>
-    <x:row r="8" ht="30" customHeight="1">
-      <x:c r="A8" s="20" t="str">
-        <x:v>聚合酶 Mix II（E2）†</x:v>
-      </x:c>
-      <x:c r="B8" s="20" t="str">
+    <x:row r="8" ht="45" customHeight="1">
+      <x:c r="A8" s="40" t="str">
+        <x:v>DNB聚合酶混合液Ⅱ（LC）</x:v>
+      </x:c>
+      <x:c r="B8" s="40" t="str">
         <x:v>0.5 mL冻存管</x:v>
       </x:c>
-      <x:c r="C8" s="20" t="str">
+      <x:c r="C8" s="40" t="str">
         <x:v>POS17 C2R5</x:v>
       </x:c>
-      <x:c r="D8" s="20" t="str">
+      <x:c r="D8" s="40" t="str">
         <x:v>按SOP表10-1手工分装</x:v>
       </x:c>
-      <x:c r="E8" s="34" t="n">
+      <x:c r="E8" s="41" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="F8" s="34" t="n">
+      <x:c r="F8" s="41" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="G8" s="34" t="n">
+      <x:c r="G8" s="41" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="H8" s="34"/>
     </x:row>
-    <x:row r="9" ht="30" customHeight="1">
-      <x:c r="A9" s="20" t="str">
+    <x:row r="9" ht="45" customHeight="1">
+      <x:c r="A9" s="40" t="str">
         <x:v>DNB终止缓冲液</x:v>
       </x:c>
-      <x:c r="B9" s="20" t="str">
+      <x:c r="B9" s="40" t="str">
         <x:v>0.5 mL冻存管</x:v>
       </x:c>
-      <x:c r="C9" s="20" t="str">
+      <x:c r="C9" s="40" t="str">
         <x:v>POS17 C4R5</x:v>
       </x:c>
-      <x:c r="D9" s="20" t="str">
+      <x:c r="D9" s="40" t="str">
         <x:v>按SOP表10-1</x:v>
       </x:c>
-      <x:c r="E9" s="34" t="n">
+      <x:c r="E9" s="41" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="F9" s="34" t="n">
+      <x:c r="F9" s="41" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="G9" s="34" t="n">
+      <x:c r="G9" s="41" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="H9" s="34"/>
     </x:row>
-    <x:row r="10" ht="30" customHeight="1">
-      <x:c r="A10" s="20"/>
-      <x:c r="B10" s="20"/>
-      <x:c r="C10" s="20"/>
-      <x:c r="D10" s="20"/>
-      <x:c r="E10" s="34"/>
-      <x:c r="F10" s="34"/>
-      <x:c r="G10" s="34"/>
-      <x:c r="H10" s="34"/>
+    <x:row r="10" ht="85" customHeight="1">
+      <x:c r="A10" s="40" t="str">
+        <x:v>T2溶解液</x:v>
+      </x:c>
+      <x:c r="B10" s="40" t="str">
+        <x:v>8 mL管（用后回收，须盖黑色胶塞）</x:v>
+      </x:c>
+      <x:c r="C10" s="40" t="str">
+        <x:v>POS24 C1R2</x:v>
+      </x:c>
+      <x:c r="D10" s="40" t="str">
+        <x:v>仅上机前准备需配；全流程见SOP表9</x:v>
+      </x:c>
+      <x:c r="E10" s="41" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="F10" s="41" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="G10" s="41" t="n">
+        <x:v>6000</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>